<commit_message>
Document the UX conventions; refresh README screenshots and example exports
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -1,27 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Checks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Findings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Licences" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Data freshness" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data freshness" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Checks'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$138</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Licences'!$A$1:$J$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Licences'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$26</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$28</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Data freshness'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 4 Oct 2026, 21:07 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 9 Oct 2026, 16:42 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>31% on 6 Sep 2026</t>
+          <t>31% on 11 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>45.3% on 6 Sep 2026</t>
+          <t>45.3% on 11 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4 on 6 Sep 2026</t>
+          <t>4 on 11 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>52 on 6 Sep 2026</t>
+          <t>52 on 11 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C15" s="7" t="n"/>
     </row>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F54"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2408,8 +2408,35 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>No accounts are at risk in Entra ID Protection</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Risky users need Entra ID P2</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Check each account with the person. If they don't recognise recent sign-ins, reset the password, sign them out everywhere (revoke sessions), and check their MFA methods, inbox rules and app consents; then confirm the account compromised or dismiss the risk in Entra ID Protection. Add a Conditional Access policy that asks for a secure password change on high user risk. The Risky users report lists each account.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F54"/>
+  <autoFilter ref="A1:F55"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -4269,7 +4296,7 @@
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 2 Oct 2026</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 7 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4335,7 +4362,7 @@
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 15 Apr 2026</t>
+          <t>Licensed member, last signed in 20 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -4357,7 +4384,7 @@
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 27 Feb 2026</t>
+          <t>Licensed member, last signed in 4 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -4379,7 +4406,7 @@
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 27 May 2026</t>
+          <t>Licensed member, last signed in 1 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -4401,7 +4428,7 @@
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 30 Jan 2026</t>
+          <t>Licensed member, last signed in 4 Feb 2026</t>
         </is>
       </c>
     </row>
@@ -4423,7 +4450,7 @@
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 28 May 2026</t>
+          <t>Licensed member, last signed in 2 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -4445,7 +4472,7 @@
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 1 Jul 2026</t>
+          <t>Licensed member, last signed in 6 Jul 2026</t>
         </is>
       </c>
     </row>
@@ -5725,7 +5752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C26"/>
+  <dimension ref="A1:C28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5757,7 +5784,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5772,7 +5799,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5787,7 +5814,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5802,7 +5829,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5817,7 +5844,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5832,7 +5859,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5847,7 +5874,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5862,7 +5889,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5877,7 +5904,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5892,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5907,7 +5934,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5922,7 +5949,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5937,7 +5964,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5948,11 +5975,11 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Mailboxes</t>
+          <t>Deleted users and groups</t>
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5963,11 +5990,11 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Inbox rules</t>
+          <t>Mailboxes</t>
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46299.8794212963</v>
+        <v>46304.69524305555</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -5978,11 +6005,11 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Mailbox size</t>
+          <t>Inbox rules</t>
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -5993,11 +6020,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Legacy sign-ins</t>
+          <t>Mailbox size</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6008,11 +6035,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sign-in activity</t>
+          <t>Legacy sign-ins</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6023,11 +6050,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Email domains</t>
+          <t>Sign-in activity</t>
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6038,11 +6065,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Devices</t>
+          <t>Risky users</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6053,11 +6080,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Directory sync</t>
+          <t>Email domains</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6068,11 +6095,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive usage</t>
+          <t>Devices</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6083,11 +6110,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Shared files</t>
+          <t>Directory sync</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6098,11 +6125,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SharePoint storage</t>
+          <t>SharePoint and OneDrive usage</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46299.87943287037</v>
+        <v>46304.69525462963</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6113,20 +6140,50 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>Shared files</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="n">
+        <v>46304.69525462963</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>SharePoint storage</t>
+        </is>
+      </c>
+      <c r="B27" s="12" t="n">
+        <v>46304.69525462963</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
           <t>Microsoft 365 usage</t>
         </is>
       </c>
-      <c r="B26" s="12" t="n">
-        <v>46299.87943287037</v>
-      </c>
-      <c r="C26" t="inlineStr">
+      <c r="B28" s="12" t="n">
+        <v>46304.69525462963</v>
+      </c>
+      <c r="C28" t="inlineStr">
         <is>
           <t>Up to date</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:C26"/>
+  <autoFilter ref="A1:C28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Sample reports that add up, and clearer website wording
The monthly review's What changed now lists the new or returning findings it counts, with the tenant's own
changes under their own heading, so "14 new" sits above 14 listed items. Terabytes show two decimals so
used, free and total agree on the SharePoint storage report, and the demo's libraries leave room for each
site's recycle bin so the storage parts add up to what's used. test_demo_samples checks both on the demo
data that makes the examples, screenshots and public demo, which are regenerated here.

The website says read-only applies to client tenants and that email goes out through the MSP's own mail
server or a separate send-only app; calls the project free software with the source coming until the
repository is public; and shows Get in touch and Ask for early access when OFFICESENTRY_WEBSITE_CONTACT
is set.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Checks" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Findings" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Licences" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data freshness" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Checks" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Findings" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Licences" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Data freshness" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 16:42 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 9 Oct 2026, 23:19 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -1258,7 +1258,7 @@
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>All 3 shared mailbox(es) block sign-in</t>
+          <t>All 3 shared mailboxes block sign-in</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -5032,7 +5032,7 @@
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.9 GB older versions</t>
+          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5059,7 +5059,7 @@
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>483.2 GB, of which 46.0 GB in the recycle bin and 36.8 GB older versions</t>
+          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5086,7 +5086,7 @@
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>65.3 GB, of which 1.0 GB in the recycle bin and 5.0 GB older versions</t>
+          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5113,7 +5113,7 @@
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>352.6 GB, of which 12.0 GB in the recycle bin and 26.2 GB older versions</t>
+          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5140,7 +5140,7 @@
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.6 GB older versions</t>
+          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5859,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97091435185</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.69524305555</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6009,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6020,11 +6020,11 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Mailbox size</t>
+          <t>Sign-in activity</t>
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6035,11 +6035,11 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Legacy sign-ins</t>
+          <t>Mailbox size</t>
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6050,11 +6050,11 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Sign-in activity</t>
+          <t>Legacy sign-ins</t>
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6099,7 +6099,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46304.69525462963</v>
+        <v>46304.97092592593</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Regenerate the examples and screenshot baselines on the merged branch
The monthly review and SharePoint storage baselines show the new change list and terabyte figures. System
status shows the database version from the activity history and precomputed rows migrations.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 23:19 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 9 Oct 2026, 23:28 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5859,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.97091435185</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6009,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6024,7 +6024,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6099,7 +6099,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46304.97092592593</v>
+        <v>46304.97725694445</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Website: retake screenshots on every deploy, and show tonight's new pages
The Deploy workflow now runs scripts/screenshots.py before building the website, so its screenshots and
example reports always show the code being deployed, new pages included, with nothing to commit. If that
step fails, the site uses the copies in the repository.

New shots and front-page cards for Coming up, Activity history, Tenant groups and System status. The demo
data gains three tenant groups, so the group picker and the public demo show them. The screenshot site
records last night's backups and a roomy disk, so System status shows a looked-after server. The examples,
README screenshots and the UI baselines those groups change are regenerated.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 23:28 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 9 Oct 2026, 23:46 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5859,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6009,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6024,7 +6024,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6099,7 +6099,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46304.97725694445</v>
+        <v>46304.99011574074</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Website: hello@officesentry.co.uk for Get in touch, and images retaken on current main
The project's own site uses hello@officesentry.co.uk for Get in touch and Ask for early access unless the
OFFICESENTRY_WEBSITE_CONTACT variable says otherwise. The examples and README screenshots are retaken on
main with the batch that merged tonight.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 23:46 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 9 Oct 2026, 23:53 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -5784,7 +5784,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5799,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5814,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5829,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5844,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5859,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5874,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5889,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5904,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5919,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5934,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5949,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5964,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +5979,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +5994,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6009,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6024,7 +6024,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6039,7 +6039,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99449074074</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6054,7 +6054,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6069,7 +6069,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6084,7 +6084,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6099,7 +6099,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6114,7 +6114,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6129,7 +6129,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6144,7 +6144,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6159,7 +6159,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6174,7 +6174,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46304.99011574074</v>
+        <v>46304.99450231482</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Say "clients" for the companies you look after, "tenant" only for Microsoft 365
Menus, page titles, buttons, emails, PDFs, spreadsheets and the docs now say client where they
said tenant. Tenants is Clients, All tenants is All clients, Client tenants is Client settings,
Tenant groups is Client groups, and the account manager's home page is Accounts. Saved views
that filter on the old Tenant column keep working.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -17,11 +17,11 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Checks'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$139</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Licences'!$A$1:$J$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Licences'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Data freshness'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 23:53 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 10 Oct 2026, 20:56 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>31% on 11 Sep 2026</t>
+          <t>33% on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>45.3% on 11 Sep 2026</t>
+          <t>46.9% on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4 on 11 Sep 2026</t>
+          <t>4 on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>52 on 11 Sep 2026</t>
+          <t>52 on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -630,11 +630,11 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1 critical, 25 high, 53 medium, 58 low findings</t>
+          <t>1 critical, 26 high, 53 medium, 58 low findings</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="7" t="n"/>
     </row>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
@@ -943,12 +943,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>No guest holds a privileged role</t>
+          <t>1 guest admin assignment</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2456,7 +2461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2567,17 +2572,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1 app with access to mail, files or the directory</t>
+          <t>1 guest admin assignment</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mail Sync Pro</t>
+          <t>g#EXT#@fabrikam.example</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Mail.Read (application permission; unverified publisher)</t>
+          <t>Guest holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -2589,17 +2594,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 computers not encrypted</t>
+          <t>1 app with access to mail, files or the directory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>Mail Sync Pro</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Windows disk isn't encrypted</t>
+          <t>Mail.Read (application permission; unverified publisher)</t>
         </is>
       </c>
     </row>
@@ -2616,17 +2621,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Windows disk isn't encrypted</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2643,12 +2643,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Windows disk isn't encrypted</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2670,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -2687,7 +2692,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -2709,7 +2714,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -2726,17 +2731,17 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>7 of 54 Windows computers past end of support</t>
+          <t>6 of 54 computers not encrypted</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LAPTOP-HARRIS31 (noah.harris@fabrikam.example)</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Windows 10 stopped getting security updates on 14 Oct 2025. Extended Security Updates or LTSC can cover it; otherwise upgrade.</t>
+          <t>Windows disk isn't encrypted</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2758,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LAPTOP-JACKSON49 (chloe.jackson@fabrikam.example)</t>
+          <t>LAPTOP-HARRIS31 (noah.harris@fabrikam.example)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -2775,7 +2780,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-JACKSON49 (chloe.jackson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -2797,7 +2802,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LAPTOP-SMITH13 (owen.smith@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2819,7 +2824,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LAPTOP-WALKER04 (rhys.walker@fabrikam.example)</t>
+          <t>LAPTOP-SMITH13 (owen.smith@fabrikam.example)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -2841,7 +2846,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WALKER04 (rhys.walker@fabrikam.example)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2863,7 +2868,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LAPTOP-WOOD22 (william.wood@fabrikam.example)</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -2875,7 +2880,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -2885,12 +2890,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DESK-ALLEN09 (thomas.allen@fabrikam.example)</t>
+          <t>LAPTOP-WOOD22 (william.wood@fabrikam.example)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+          <t>Windows 10 stopped getting security updates on 14 Oct 2025. Extended Security Updates or LTSC can cover it; otherwise upgrade.</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2912,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DESK-CLARK06 (ruby.clark@fabrikam.example)</t>
+          <t>DESK-ALLEN09 (thomas.allen@fabrikam.example)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -2929,7 +2934,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DESK-HARRISON21 (leo.harrison@fabrikam.example)</t>
+          <t>DESK-CLARK06 (ruby.clark@fabrikam.example)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2951,7 +2956,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DESK-KHAN30 (owen.khan@fabrikam.example)</t>
+          <t>DESK-HARRISON21 (leo.harrison@fabrikam.example)</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2973,7 +2978,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DESK-KING24 (megan.king@fabrikam.example)</t>
+          <t>DESK-KHAN30 (owen.khan@fabrikam.example)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2995,7 +3000,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>DESK-KING24 (megan.king@fabrikam.example)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -3017,7 +3022,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DESK-ROBERTS45 (jack.roberts@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -3039,17 +3044,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-ROBERTS45 (jack.roberts@fabrikam.example)</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3066,12 +3066,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DESK-WHITE42 (lily.white@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3093,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DESK-WILLIAMS27 (arthur.williams@fabrikam.example)</t>
+          <t>DESK-WHITE42 (lily.white@fabrikam.example)</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -3110,7 +3115,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DESK-WOOD39 (ruby.wood@fabrikam.example)</t>
+          <t>DESK-WILLIAMS27 (arthur.williams@fabrikam.example)</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -3132,7 +3137,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LAPTOP-BROWN01 (aisha.brown@fabrikam.example)</t>
+          <t>DESK-WOOD39 (ruby.wood@fabrikam.example)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -3154,7 +3159,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>LAPTOP-BROWN01 (aisha.brown@fabrikam.example)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3176,7 +3181,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LAPTOP-GREEN32 (megan.green@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -3198,7 +3203,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LAPTOP-JOHNSON47 (thomas.johnson@fabrikam.example)</t>
+          <t>LAPTOP-GREEN32 (megan.green@fabrikam.example)</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -3220,7 +3225,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LAPTOP-JONES34 (ethan.jones@fabrikam.example)</t>
+          <t>LAPTOP-JOHNSON47 (thomas.johnson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -3242,7 +3247,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LAPTOP-KHAN35 (lily.khan@fabrikam.example)</t>
+          <t>LAPTOP-JONES34 (ethan.jones@fabrikam.example)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -3264,7 +3269,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE02 (jack.lee@fabrikam.example)</t>
+          <t>LAPTOP-KHAN35 (lily.khan@fabrikam.example)</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -3286,7 +3291,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-LEE02 (jack.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -3308,7 +3313,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBERTS41 (henry.roberts@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -3330,7 +3335,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LAPTOP-SCOTT17 (owen.scott@fabrikam.example)</t>
+          <t>LAPTOP-ROBERTS41 (henry.roberts@fabrikam.example)</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -3352,7 +3357,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LAPTOP-SCOTT19 (isla.scott@fabrikam.example)</t>
+          <t>LAPTOP-SCOTT17 (owen.scott@fabrikam.example)</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -3374,17 +3379,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LAPTOP-SMITH50 (oscar.smith@fabrikam.example)</t>
+          <t>LAPTOP-SCOTT19 (isla.scott@fabrikam.example)</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LAPTOP-TAYLOR43 (olivia.taylor@fabrikam.example)</t>
+          <t>LAPTOP-SMITH50 (oscar.smith@fabrikam.example)</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3428,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LAPTOP-THOMAS08 (ava.thomas@fabrikam.example)</t>
+          <t>LAPTOP-TAYLOR43 (olivia.taylor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -3445,7 +3450,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LAPTOP-TURNER37 (callum.turner@fabrikam.example)</t>
+          <t>LAPTOP-THOMAS08 (ava.thomas@fabrikam.example)</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -3467,7 +3472,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LAPTOP-WALKER10 (george.walker@fabrikam.example)</t>
+          <t>LAPTOP-TURNER37 (callum.turner@fabrikam.example)</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -3489,7 +3494,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-WALKER10 (george.walker@fabrikam.example)</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -3511,7 +3516,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LAPTOP-WILLIAMS20 (priya.williams@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -3523,22 +3528,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>1 suspicious inbox rule</t>
+          <t>7 of 54 Windows computers past end of support</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>LAPTOP-WILLIAMS20 (priya.williams@fabrikam.example)</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>".": Moves to RSS Feeds mail mentioning invoice, payment; Rule name '.' looks deliberately blank</t>
+          <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3555,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>5 external forwards</t>
+          <t>1 suspicious inbox rule</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3560,7 +3565,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to anna.kowalski@homemail.example (keeps a copy)</t>
+          <t>".": Moves to RSS Feeds mail mentioning invoice, payment; Rule name '.' looks deliberately blank</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3587,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Inbox rule "Copy to home" forwards to anna.kowalski.home@homemail.example</t>
+          <t>Mailbox forwarding to anna.kowalski@homemail.example (keeps a copy)</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3604,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>rhys.hall@fabrikam.example</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to rhys.hall@homemail.example (doesn't keep a copy)</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Inbox rule "Copy to home" forwards to anna.kowalski.home@homemail.example</t>
         </is>
       </c>
     </row>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>rhys.hall@fabrikam.example</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to rhys.walker@homemail.example (doesn't keep a copy)</t>
+          <t>Mailbox forwarding to rhys.hall@homemail.example (doesn't keep a copy)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3653,12 +3653,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>thomas.robinson@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Inbox rule "Invoices to bookkeeper" forwards to bookkeeping@ledgerline.example</t>
+          <t>Mailbox forwarding to rhys.walker@homemail.example (doesn't keep a copy)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3670,24 +3675,24 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>5 external forwards</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>thomas.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>No MFA method registered</t>
+          <t>Inbox rule "Invoices to bookkeeper" forwards to bookkeeping@ledgerline.example</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -3697,7 +3702,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -3719,7 +3724,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -3741,7 +3746,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>amelia.khan@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -3763,7 +3768,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>arthur.williams@fabrikam.example</t>
+          <t>amelia.khan@fabrikam.example</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -3785,7 +3790,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ava.jackson@fabrikam.example</t>
+          <t>arthur.williams@fabrikam.example</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -3807,7 +3812,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ava.moore@fabrikam.example</t>
+          <t>ava.jackson@fabrikam.example</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -3829,7 +3834,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ava.thomas@fabrikam.example</t>
+          <t>ava.moore@fabrikam.example</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -3851,7 +3856,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>carl.svensson@fabrikam.example</t>
+          <t>ava.thomas@fabrikam.example</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3873,7 +3878,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>chloe.jackson@fabrikam.example</t>
+          <t>carl.svensson@fabrikam.example</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -3895,7 +3900,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>george.williams@fabrikam.example</t>
+          <t>chloe.jackson@fabrikam.example</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -3917,7 +3922,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>henry.roberts@fabrikam.example</t>
+          <t>george.williams@fabrikam.example</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -3939,7 +3944,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>isla.scott@fabrikam.example</t>
+          <t>henry.roberts@fabrikam.example</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3961,7 +3966,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>isla.scott@fabrikam.example</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -3983,7 +3988,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>jack.roberts@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -4005,7 +4010,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>lily.khan@fabrikam.example</t>
+          <t>jack.roberts@fabrikam.example</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -4027,7 +4032,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>lily.watson@fabrikam.example</t>
+          <t>lily.khan@fabrikam.example</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -4049,7 +4054,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>lily.white@fabrikam.example</t>
+          <t>lily.watson@fabrikam.example</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -4071,7 +4076,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>megan.king@fabrikam.example</t>
+          <t>lily.white@fabrikam.example</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -4093,7 +4098,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>megan.king@fabrikam.example</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -4115,7 +4120,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>olivia.taylor@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -4137,7 +4142,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>owen.scott@fabrikam.example</t>
+          <t>olivia.taylor@fabrikam.example</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -4159,7 +4164,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>owen.scott@fabrikam.example</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -4181,7 +4186,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ruby.davies@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -4203,7 +4208,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ruby.wood@fabrikam.example</t>
+          <t>ruby.davies@fabrikam.example</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -4225,7 +4230,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>thomas.johnson@fabrikam.example</t>
+          <t>ruby.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -4247,7 +4252,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>thomas.johnson@fabrikam.example</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -4259,22 +4264,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Legacy authentication is allowed</t>
+          <t>27 users without MFA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>No enabled policy blocks legacy authentication for all users</t>
+          <t>No MFA method registered</t>
         </is>
       </c>
     </row>
@@ -4286,17 +4291,17 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>1 domain had sign-in settings changed in the last 30 days</t>
+          <t>Legacy authentication is allowed</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 7 Oct 2026</t>
+          <t>No enabled policy blocks legacy authentication for all users</t>
         </is>
       </c>
     </row>
@@ -4308,24 +4313,24 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>1 domain had sign-in settings changed in the last 30 days</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clients (Finance / Documents)</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Anyone can edit, link never expires</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 8 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4335,12 +4340,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
+          <t>Clients (Finance / Documents)</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>Anyone can view</t>
+          <t>Anyone can edit, link never expires</t>
         </is>
       </c>
     </row>
@@ -4352,17 +4357,17 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 20 Apr 2026</t>
+          <t>Anyone can view</t>
         </is>
       </c>
     </row>
@@ -4379,12 +4384,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 4 Mar 2026</t>
+          <t>Licensed member, last signed in 21 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -4401,12 +4406,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 1 Jun 2026</t>
+          <t>Licensed member, last signed in 5 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -4423,12 +4428,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 4 Feb 2026</t>
+          <t>Licensed member, last signed in 2 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -4445,12 +4450,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 2 Jun 2026</t>
+          <t>Licensed member, last signed in 5 Feb 2026</t>
         </is>
       </c>
     </row>
@@ -4467,19 +4472,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 6 Jul 2026</t>
+          <t>Licensed member, last signed in 3 Jun 2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4489,34 +4494,34 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Member, never signed in, created ?</t>
+          <t>Licensed member, last signed in 7 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>7 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>g#EXT#@fabrikam.example</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with Authenticator app</t>
+          <t>Guest, never signed in, created ?</t>
         </is>
       </c>
     </row>
@@ -4533,12 +4538,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with no MFA method at all</t>
+          <t>Global Administrator; signs in with Authenticator app</t>
         </is>
       </c>
     </row>
@@ -4550,17 +4555,17 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>1 app with privileged roles</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Some app</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>App holding Exchange Administrator</t>
+          <t>Global Administrator; signs in with no MFA method at all</t>
         </is>
       </c>
     </row>
@@ -4572,17 +4577,17 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Users can consent to any app</t>
+          <t>1 app with privileged roles</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>Some app</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Any user can grant any app access to their mail and files</t>
+          <t>App holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -4594,17 +4599,17 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>Users can consent to any app</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>Any user can grant any app access to their mail and files</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4626,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -4643,17 +4648,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4670,12 +4670,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4697,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4714,7 +4719,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4736,7 +4741,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4758,7 +4763,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4780,7 +4785,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4797,17 +4802,17 @@
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>1 mail domain without DKIM</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4824,7 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>1 mail domain without DKIM</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4829,14 +4834,14 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
+          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -4846,41 +4851,41 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no DMARC p=reject record</t>
+          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Project Phoenix</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Team, only owner is disabled (Ben Okafor)</t>
+          <t>Doesn't receive mail but has no DMARC p=reject record</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -4890,12 +4895,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Project Phoenix</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, no owner</t>
+          <t>Team, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
@@ -4912,34 +4917,34 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Provisioned</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
+          <t>Microsoft 365 group, no owner</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
+          <t>3 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>Provisioned</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>Excluded from "Require MFA for all users"</t>
+          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
         </is>
       </c>
     </row>
@@ -4951,17 +4956,17 @@
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>1 disabled account still licensed</t>
+          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ben.okafor@fabrikam.example</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>Disabled, holding 1 licence</t>
+          <t>Excluded from "Require MFA for all users"</t>
         </is>
       </c>
     </row>
@@ -4973,17 +4978,17 @@
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including anonymous links</t>
+          <t>1 disabled account still licensed</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive</t>
+          <t>ben.okafor@fabrikam.example</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>Anyone links are allowed</t>
+          <t>Disabled, holding 1 licence</t>
         </is>
       </c>
     </row>
@@ -4995,29 +5000,24 @@
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>Anyone, including anonymous links</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Tenant SharePoint storage</t>
+          <t>SharePoint and OneDrive</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone links are allowed</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -5027,12 +5027,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/finance</t>
+          <t>Tenant SharePoint storage</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5054,12 +5054,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
+          <t>https://fabrikam.sharepoint.com/sites/finance</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
+          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
+          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
+          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5108,12 +5108,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
+          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
+          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5135,12 +5135,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/practice</t>
+          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5157,17 +5157,22 @@
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>1 app registration with expiring or expired credentials</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Old connector</t>
+          <t>https://fabrikam.sharepoint.com/sites/practice</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>The 1 credential expired, last on 1 Jan 2025</t>
+          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5179,17 +5184,17 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>1 of 55 joined computers not in Intune</t>
+          <t>1 app registration with expiring or expired credentials</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>DESK-RECEPTION</t>
+          <t>Old connector</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>Hybrid joined, not managed by Intune</t>
+          <t>The 1 credential expired, last on 1 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -5201,17 +5206,17 @@
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 of 55 joined computers not in Intune</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>DESK-RECEPTION</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>Hybrid joined, not managed by Intune</t>
         </is>
       </c>
     </row>
@@ -5228,17 +5233,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
           <t>Last check-in 38 days ago</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5255,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
           <t>Last check-in 38 days ago</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5282,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
@@ -5299,12 +5304,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 45 days ago</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -5316,17 +5321,17 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>1 of 57 device records unused for 90+ days</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>OLD-PC</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Windows, last seen 200 days ago</t>
+          <t>Last check-in 45 days ago</t>
         </is>
       </c>
     </row>
@@ -5338,17 +5343,17 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>1 domain with SPF problems</t>
+          <t>1 of 57 device records unused for 90+ days</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>OLD-PC</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
+          <t>Windows, last seen 200 days ago</t>
         </is>
       </c>
     </row>
@@ -5360,17 +5365,17 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
+          <t>1 domain with SPF problems</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
+          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
         </is>
       </c>
     </row>
@@ -5382,17 +5387,17 @@
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is on for the organisation</t>
+          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is allowed</t>
+          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
         </is>
       </c>
     </row>
@@ -5404,7 +5409,7 @@
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including guests, can invite guests</t>
+          <t>SMTP AUTH is on for the organisation</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5414,7 +5419,7 @@
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>Guests can invite other guests</t>
+          <t>SMTP AUTH is allowed</t>
         </is>
       </c>
     </row>
@@ -5426,17 +5431,17 @@
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>Anyone, including guests, can invite guests</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>george.baker@fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>Guests can invite other guests</t>
         </is>
       </c>
     </row>
@@ -5453,17 +5458,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>owen.robinson@fabrikam.example</t>
+          <t>george.baker@fabrikam.example</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
           <t>Second factor is only Mobile phone (SMS or call)</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5480,17 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>owen.turner@fabrikam.example</t>
+          <t>owen.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
           <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5507,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>thomas.allen@fabrikam.example</t>
+          <t>owen.turner@fabrikam.example</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
@@ -5519,17 +5524,17 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>4 people can only use a text or call as a second factor</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Basic</t>
+          <t>thomas.allen@fabrikam.example</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
         </is>
       </c>
     </row>
@@ -5546,12 +5551,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Premium</t>
+          <t>Microsoft 365 Business Basic</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+          <t>2 of 13 unassigned, 9.80 GBP/month</t>
         </is>
       </c>
     </row>
@@ -5563,22 +5568,44 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Premium</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
           <t>Any user can register an app</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>Whole organisation</t>
         </is>
       </c>
-      <c r="D138" s="7" t="inlineStr">
+      <c r="D139" s="7" t="inlineStr">
         <is>
           <t>Users can register apps that nobody reviews</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E138"/>
+  <autoFilter ref="A1:E139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -5752,7 +5779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5784,7 +5811,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5826,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5841,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5856,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5871,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5886,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5901,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5916,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5931,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5946,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5961,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5976,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5991,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +6006,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +6021,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6036,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6024,7 +6051,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6039,7 +6066,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6054,7 +6081,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6065,11 +6092,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Risky users</t>
+          <t>Mobile devices</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6080,11 +6107,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Email domains</t>
+          <t>Automatic replies</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6095,11 +6122,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Devices</t>
+          <t>Distribution lists</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6110,11 +6137,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Directory sync</t>
+          <t>Risky users</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6125,11 +6152,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive usage</t>
+          <t>Email domains</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6140,11 +6167,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Shared files</t>
+          <t>Devices</t>
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6155,11 +6182,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SharePoint storage</t>
+          <t>Directory sync</t>
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6170,20 +6197,110 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>SharePoint and OneDrive usage</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Shared files</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SharePoint storage</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Microsoft 365 usage</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n">
-        <v>46304.99450231482</v>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B31" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>Up to date</t>
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>App sign-ins</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Group nesting</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Departments and managers</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C28"/>
+  <autoFilter ref="A1:C34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Say "clients" for the companies you look after, "tenant" only for Microsoft 365 (#11)
Wording only: menus, pages, emails, exports, docs and website say client; tenant stays for the Microsoft 365 side. Saved views on the old column names still work.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -17,11 +17,11 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$55</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Checks'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$139</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Licences'!$A$1:$J$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Licences'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$28</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$34</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Data freshness'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 9 Oct 2026, 23:53 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 10 Oct 2026, 20:56 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>31% on 11 Sep 2026</t>
+          <t>33% on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>45.3% on 11 Sep 2026</t>
+          <t>46.9% on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4 on 11 Sep 2026</t>
+          <t>4 on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>52 on 11 Sep 2026</t>
+          <t>52 on 12 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -630,11 +630,11 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1 critical, 25 high, 53 medium, 58 low findings</t>
+          <t>1 critical, 26 high, 53 medium, 58 low findings</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C14" s="7" t="n"/>
     </row>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>27</v>
+        <v>33</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
@@ -943,12 +943,17 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>No guest holds a privileged role</t>
+          <t>1 guest admin assignment</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -2456,7 +2461,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E138"/>
+  <dimension ref="A1:E139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2567,17 +2572,17 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1 app with access to mail, files or the directory</t>
+          <t>1 guest admin assignment</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Mail Sync Pro</t>
+          <t>g#EXT#@fabrikam.example</t>
         </is>
       </c>
       <c r="D5" s="7" t="inlineStr">
         <is>
-          <t>Mail.Read (application permission; unverified publisher)</t>
+          <t>Guest holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -2589,17 +2594,17 @@
       </c>
       <c r="B6" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 computers not encrypted</t>
+          <t>1 app with access to mail, files or the directory</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>Mail Sync Pro</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>Windows disk isn't encrypted</t>
+          <t>Mail.Read (application permission; unverified publisher)</t>
         </is>
       </c>
     </row>
@@ -2616,17 +2621,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Windows disk isn't encrypted</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2643,12 +2643,17 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D8" s="7" t="inlineStr">
         <is>
           <t>Windows disk isn't encrypted</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -2665,7 +2670,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D9" s="7" t="inlineStr">
@@ -2687,7 +2692,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D10" s="7" t="inlineStr">
@@ -2709,7 +2714,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D11" s="7" t="inlineStr">
@@ -2726,17 +2731,17 @@
       </c>
       <c r="B12" s="7" t="inlineStr">
         <is>
-          <t>7 of 54 Windows computers past end of support</t>
+          <t>6 of 54 computers not encrypted</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>LAPTOP-HARRIS31 (noah.harris@fabrikam.example)</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>Windows 10 stopped getting security updates on 14 Oct 2025. Extended Security Updates or LTSC can cover it; otherwise upgrade.</t>
+          <t>Windows disk isn't encrypted</t>
         </is>
       </c>
     </row>
@@ -2753,7 +2758,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>LAPTOP-JACKSON49 (chloe.jackson@fabrikam.example)</t>
+          <t>LAPTOP-HARRIS31 (noah.harris@fabrikam.example)</t>
         </is>
       </c>
       <c r="D13" s="7" t="inlineStr">
@@ -2775,7 +2780,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-JACKSON49 (chloe.jackson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D14" s="7" t="inlineStr">
@@ -2797,7 +2802,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>LAPTOP-SMITH13 (owen.smith@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D15" s="7" t="inlineStr">
@@ -2819,7 +2824,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>LAPTOP-WALKER04 (rhys.walker@fabrikam.example)</t>
+          <t>LAPTOP-SMITH13 (owen.smith@fabrikam.example)</t>
         </is>
       </c>
       <c r="D16" s="7" t="inlineStr">
@@ -2841,7 +2846,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WALKER04 (rhys.walker@fabrikam.example)</t>
         </is>
       </c>
       <c r="D17" s="7" t="inlineStr">
@@ -2863,7 +2868,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>LAPTOP-WOOD22 (william.wood@fabrikam.example)</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D18" s="7" t="inlineStr">
@@ -2875,7 +2880,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
@@ -2885,12 +2890,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>DESK-ALLEN09 (thomas.allen@fabrikam.example)</t>
+          <t>LAPTOP-WOOD22 (william.wood@fabrikam.example)</t>
         </is>
       </c>
       <c r="D19" s="7" t="inlineStr">
         <is>
-          <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+          <t>Windows 10 stopped getting security updates on 14 Oct 2025. Extended Security Updates or LTSC can cover it; otherwise upgrade.</t>
         </is>
       </c>
     </row>
@@ -2907,7 +2912,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>DESK-CLARK06 (ruby.clark@fabrikam.example)</t>
+          <t>DESK-ALLEN09 (thomas.allen@fabrikam.example)</t>
         </is>
       </c>
       <c r="D20" s="7" t="inlineStr">
@@ -2929,7 +2934,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>DESK-HARRISON21 (leo.harrison@fabrikam.example)</t>
+          <t>DESK-CLARK06 (ruby.clark@fabrikam.example)</t>
         </is>
       </c>
       <c r="D21" s="7" t="inlineStr">
@@ -2951,7 +2956,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>DESK-KHAN30 (owen.khan@fabrikam.example)</t>
+          <t>DESK-HARRISON21 (leo.harrison@fabrikam.example)</t>
         </is>
       </c>
       <c r="D22" s="7" t="inlineStr">
@@ -2973,7 +2978,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>DESK-KING24 (megan.king@fabrikam.example)</t>
+          <t>DESK-KHAN30 (owen.khan@fabrikam.example)</t>
         </is>
       </c>
       <c r="D23" s="7" t="inlineStr">
@@ -2995,7 +3000,7 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>DESK-KING24 (megan.king@fabrikam.example)</t>
         </is>
       </c>
       <c r="D24" s="7" t="inlineStr">
@@ -3017,7 +3022,7 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>DESK-ROBERTS45 (jack.roberts@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D25" s="7" t="inlineStr">
@@ -3039,17 +3044,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-ROBERTS45 (jack.roberts@fabrikam.example)</t>
         </is>
       </c>
       <c r="D26" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3066,12 +3066,17 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>DESK-WHITE42 (lily.white@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3088,7 +3093,7 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>DESK-WILLIAMS27 (arthur.williams@fabrikam.example)</t>
+          <t>DESK-WHITE42 (lily.white@fabrikam.example)</t>
         </is>
       </c>
       <c r="D28" s="7" t="inlineStr">
@@ -3110,7 +3115,7 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>DESK-WOOD39 (ruby.wood@fabrikam.example)</t>
+          <t>DESK-WILLIAMS27 (arthur.williams@fabrikam.example)</t>
         </is>
       </c>
       <c r="D29" s="7" t="inlineStr">
@@ -3132,7 +3137,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LAPTOP-BROWN01 (aisha.brown@fabrikam.example)</t>
+          <t>DESK-WOOD39 (ruby.wood@fabrikam.example)</t>
         </is>
       </c>
       <c r="D30" s="7" t="inlineStr">
@@ -3154,7 +3159,7 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>LAPTOP-BROWN01 (aisha.brown@fabrikam.example)</t>
         </is>
       </c>
       <c r="D31" s="7" t="inlineStr">
@@ -3176,7 +3181,7 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LAPTOP-GREEN32 (megan.green@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D32" s="7" t="inlineStr">
@@ -3198,7 +3203,7 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LAPTOP-JOHNSON47 (thomas.johnson@fabrikam.example)</t>
+          <t>LAPTOP-GREEN32 (megan.green@fabrikam.example)</t>
         </is>
       </c>
       <c r="D33" s="7" t="inlineStr">
@@ -3220,7 +3225,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LAPTOP-JONES34 (ethan.jones@fabrikam.example)</t>
+          <t>LAPTOP-JOHNSON47 (thomas.johnson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D34" s="7" t="inlineStr">
@@ -3242,7 +3247,7 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>LAPTOP-KHAN35 (lily.khan@fabrikam.example)</t>
+          <t>LAPTOP-JONES34 (ethan.jones@fabrikam.example)</t>
         </is>
       </c>
       <c r="D35" s="7" t="inlineStr">
@@ -3264,7 +3269,7 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE02 (jack.lee@fabrikam.example)</t>
+          <t>LAPTOP-KHAN35 (lily.khan@fabrikam.example)</t>
         </is>
       </c>
       <c r="D36" s="7" t="inlineStr">
@@ -3286,7 +3291,7 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-LEE02 (jack.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D37" s="7" t="inlineStr">
@@ -3308,7 +3313,7 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBERTS41 (henry.roberts@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D38" s="7" t="inlineStr">
@@ -3330,7 +3335,7 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>LAPTOP-SCOTT17 (owen.scott@fabrikam.example)</t>
+          <t>LAPTOP-ROBERTS41 (henry.roberts@fabrikam.example)</t>
         </is>
       </c>
       <c r="D39" s="7" t="inlineStr">
@@ -3352,7 +3357,7 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>LAPTOP-SCOTT19 (isla.scott@fabrikam.example)</t>
+          <t>LAPTOP-SCOTT17 (owen.scott@fabrikam.example)</t>
         </is>
       </c>
       <c r="D40" s="7" t="inlineStr">
@@ -3374,17 +3379,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>LAPTOP-SMITH50 (oscar.smith@fabrikam.example)</t>
+          <t>LAPTOP-SCOTT19 (isla.scott@fabrikam.example)</t>
         </is>
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3401,12 +3401,17 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>LAPTOP-TAYLOR43 (olivia.taylor@fabrikam.example)</t>
+          <t>LAPTOP-SMITH50 (oscar.smith@fabrikam.example)</t>
         </is>
       </c>
       <c r="D42" s="7" t="inlineStr">
         <is>
           <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3428,7 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>LAPTOP-THOMAS08 (ava.thomas@fabrikam.example)</t>
+          <t>LAPTOP-TAYLOR43 (olivia.taylor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D43" s="7" t="inlineStr">
@@ -3445,7 +3450,7 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>LAPTOP-TURNER37 (callum.turner@fabrikam.example)</t>
+          <t>LAPTOP-THOMAS08 (ava.thomas@fabrikam.example)</t>
         </is>
       </c>
       <c r="D44" s="7" t="inlineStr">
@@ -3467,7 +3472,7 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LAPTOP-WALKER10 (george.walker@fabrikam.example)</t>
+          <t>LAPTOP-TURNER37 (callum.turner@fabrikam.example)</t>
         </is>
       </c>
       <c r="D45" s="7" t="inlineStr">
@@ -3489,7 +3494,7 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-WALKER10 (george.walker@fabrikam.example)</t>
         </is>
       </c>
       <c r="D46" s="7" t="inlineStr">
@@ -3511,7 +3516,7 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LAPTOP-WILLIAMS20 (priya.williams@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D47" s="7" t="inlineStr">
@@ -3523,22 +3528,22 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>1 suspicious inbox rule</t>
+          <t>7 of 54 Windows computers past end of support</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>LAPTOP-WILLIAMS20 (priya.williams@fabrikam.example)</t>
         </is>
       </c>
       <c r="D48" s="7" t="inlineStr">
         <is>
-          <t>".": Moves to RSS Feeds mail mentioning invoice, payment; Rule name '.' looks deliberately blank</t>
+          <t>Windows 11 24H2: updates for Home and Pro end 13 Oct 2026.</t>
         </is>
       </c>
     </row>
@@ -3550,7 +3555,7 @@
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>5 external forwards</t>
+          <t>1 suspicious inbox rule</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -3560,7 +3565,7 @@
       </c>
       <c r="D49" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to anna.kowalski@homemail.example (keeps a copy)</t>
+          <t>".": Moves to RSS Feeds mail mentioning invoice, payment; Rule name '.' looks deliberately blank</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3587,7 @@
       </c>
       <c r="D50" s="7" t="inlineStr">
         <is>
-          <t>Inbox rule "Copy to home" forwards to anna.kowalski.home@homemail.example</t>
+          <t>Mailbox forwarding to anna.kowalski@homemail.example (keeps a copy)</t>
         </is>
       </c>
     </row>
@@ -3599,17 +3604,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>rhys.hall@fabrikam.example</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D51" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to rhys.hall@homemail.example (doesn't keep a copy)</t>
-        </is>
-      </c>
-      <c r="E51" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Inbox rule "Copy to home" forwards to anna.kowalski.home@homemail.example</t>
         </is>
       </c>
     </row>
@@ -3626,12 +3626,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>rhys.hall@fabrikam.example</t>
         </is>
       </c>
       <c r="D52" s="7" t="inlineStr">
         <is>
-          <t>Mailbox forwarding to rhys.walker@homemail.example (doesn't keep a copy)</t>
+          <t>Mailbox forwarding to rhys.hall@homemail.example (doesn't keep a copy)</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -3653,12 +3653,17 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>thomas.robinson@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D53" s="7" t="inlineStr">
         <is>
-          <t>Inbox rule "Invoices to bookkeeper" forwards to bookkeeping@ledgerline.example</t>
+          <t>Mailbox forwarding to rhys.walker@homemail.example (doesn't keep a copy)</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -3670,24 +3675,24 @@
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>5 external forwards</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>thomas.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D54" s="7" t="inlineStr">
         <is>
-          <t>No MFA method registered</t>
+          <t>Inbox rule "Invoices to bookkeeper" forwards to bookkeeping@ledgerline.example</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -3697,7 +3702,7 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D55" s="7" t="inlineStr">
@@ -3719,7 +3724,7 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D56" s="7" t="inlineStr">
@@ -3741,7 +3746,7 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>amelia.khan@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D57" s="7" t="inlineStr">
@@ -3763,7 +3768,7 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>arthur.williams@fabrikam.example</t>
+          <t>amelia.khan@fabrikam.example</t>
         </is>
       </c>
       <c r="D58" s="7" t="inlineStr">
@@ -3785,7 +3790,7 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>ava.jackson@fabrikam.example</t>
+          <t>arthur.williams@fabrikam.example</t>
         </is>
       </c>
       <c r="D59" s="7" t="inlineStr">
@@ -3807,7 +3812,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>ava.moore@fabrikam.example</t>
+          <t>ava.jackson@fabrikam.example</t>
         </is>
       </c>
       <c r="D60" s="7" t="inlineStr">
@@ -3829,7 +3834,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>ava.thomas@fabrikam.example</t>
+          <t>ava.moore@fabrikam.example</t>
         </is>
       </c>
       <c r="D61" s="7" t="inlineStr">
@@ -3851,7 +3856,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>carl.svensson@fabrikam.example</t>
+          <t>ava.thomas@fabrikam.example</t>
         </is>
       </c>
       <c r="D62" s="7" t="inlineStr">
@@ -3873,7 +3878,7 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>chloe.jackson@fabrikam.example</t>
+          <t>carl.svensson@fabrikam.example</t>
         </is>
       </c>
       <c r="D63" s="7" t="inlineStr">
@@ -3895,7 +3900,7 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>george.williams@fabrikam.example</t>
+          <t>chloe.jackson@fabrikam.example</t>
         </is>
       </c>
       <c r="D64" s="7" t="inlineStr">
@@ -3917,7 +3922,7 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>henry.roberts@fabrikam.example</t>
+          <t>george.williams@fabrikam.example</t>
         </is>
       </c>
       <c r="D65" s="7" t="inlineStr">
@@ -3939,7 +3944,7 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>isla.scott@fabrikam.example</t>
+          <t>henry.roberts@fabrikam.example</t>
         </is>
       </c>
       <c r="D66" s="7" t="inlineStr">
@@ -3961,7 +3966,7 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>isla.scott@fabrikam.example</t>
         </is>
       </c>
       <c r="D67" s="7" t="inlineStr">
@@ -3983,7 +3988,7 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>jack.roberts@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D68" s="7" t="inlineStr">
@@ -4005,7 +4010,7 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>lily.khan@fabrikam.example</t>
+          <t>jack.roberts@fabrikam.example</t>
         </is>
       </c>
       <c r="D69" s="7" t="inlineStr">
@@ -4027,7 +4032,7 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>lily.watson@fabrikam.example</t>
+          <t>lily.khan@fabrikam.example</t>
         </is>
       </c>
       <c r="D70" s="7" t="inlineStr">
@@ -4049,7 +4054,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>lily.white@fabrikam.example</t>
+          <t>lily.watson@fabrikam.example</t>
         </is>
       </c>
       <c r="D71" s="7" t="inlineStr">
@@ -4071,7 +4076,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>megan.king@fabrikam.example</t>
+          <t>lily.white@fabrikam.example</t>
         </is>
       </c>
       <c r="D72" s="7" t="inlineStr">
@@ -4093,7 +4098,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>megan.king@fabrikam.example</t>
         </is>
       </c>
       <c r="D73" s="7" t="inlineStr">
@@ -4115,7 +4120,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>olivia.taylor@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D74" s="7" t="inlineStr">
@@ -4137,7 +4142,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>owen.scott@fabrikam.example</t>
+          <t>olivia.taylor@fabrikam.example</t>
         </is>
       </c>
       <c r="D75" s="7" t="inlineStr">
@@ -4159,7 +4164,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>owen.scott@fabrikam.example</t>
         </is>
       </c>
       <c r="D76" s="7" t="inlineStr">
@@ -4181,7 +4186,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>ruby.davies@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D77" s="7" t="inlineStr">
@@ -4203,7 +4208,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>ruby.wood@fabrikam.example</t>
+          <t>ruby.davies@fabrikam.example</t>
         </is>
       </c>
       <c r="D78" s="7" t="inlineStr">
@@ -4225,7 +4230,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>thomas.johnson@fabrikam.example</t>
+          <t>ruby.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D79" s="7" t="inlineStr">
@@ -4247,7 +4252,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>thomas.johnson@fabrikam.example</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -4259,22 +4264,22 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>Legacy authentication is allowed</t>
+          <t>27 users without MFA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
         <is>
-          <t>No enabled policy blocks legacy authentication for all users</t>
+          <t>No MFA method registered</t>
         </is>
       </c>
     </row>
@@ -4286,17 +4291,17 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>1 domain had sign-in settings changed in the last 30 days</t>
+          <t>Legacy authentication is allowed</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 7 Oct 2026</t>
+          <t>No enabled policy blocks legacy authentication for all users</t>
         </is>
       </c>
     </row>
@@ -4308,24 +4313,24 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>1 domain had sign-in settings changed in the last 30 days</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Clients (Finance / Documents)</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Anyone can edit, link never expires</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 8 Oct 2026</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B84" s="7" t="inlineStr">
@@ -4335,12 +4340,12 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
+          <t>Clients (Finance / Documents)</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>Anyone can view</t>
+          <t>Anyone can edit, link never expires</t>
         </is>
       </c>
     </row>
@@ -4352,17 +4357,17 @@
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 20 Apr 2026</t>
+          <t>Anyone can view</t>
         </is>
       </c>
     </row>
@@ -4379,12 +4384,12 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 4 Mar 2026</t>
+          <t>Licensed member, last signed in 21 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -4401,12 +4406,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 1 Jun 2026</t>
+          <t>Licensed member, last signed in 5 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -4423,12 +4428,12 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 4 Feb 2026</t>
+          <t>Licensed member, last signed in 2 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -4445,12 +4450,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 2 Jun 2026</t>
+          <t>Licensed member, last signed in 5 Feb 2026</t>
         </is>
       </c>
     </row>
@@ -4467,19 +4472,19 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 6 Jul 2026</t>
+          <t>Licensed member, last signed in 3 Jun 2026</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
@@ -4489,34 +4494,34 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Member, never signed in, created ?</t>
+          <t>Licensed member, last signed in 7 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>7 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>g#EXT#@fabrikam.example</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with Authenticator app</t>
+          <t>Guest, never signed in, created ?</t>
         </is>
       </c>
     </row>
@@ -4533,12 +4538,12 @@
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with no MFA method at all</t>
+          <t>Global Administrator; signs in with Authenticator app</t>
         </is>
       </c>
     </row>
@@ -4550,17 +4555,17 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>1 app with privileged roles</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Some app</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>App holding Exchange Administrator</t>
+          <t>Global Administrator; signs in with no MFA method at all</t>
         </is>
       </c>
     </row>
@@ -4572,17 +4577,17 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>Users can consent to any app</t>
+          <t>1 app with privileged roles</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>Some app</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Any user can grant any app access to their mail and files</t>
+          <t>App holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -4594,17 +4599,17 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>Users can consent to any app</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>Any user can grant any app access to their mail and files</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4626,7 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
@@ -4643,17 +4648,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
-        </is>
-      </c>
-      <c r="E98" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4670,12 +4670,17 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4692,7 +4697,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4714,7 +4719,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4736,7 +4741,7 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
@@ -4758,7 +4763,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4780,7 +4785,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4797,17 +4802,17 @@
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>1 mail domain without DKIM</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -4819,7 +4824,7 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>1 mail domain without DKIM</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
@@ -4829,14 +4834,14 @@
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
+          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B107" s="7" t="inlineStr">
@@ -4846,41 +4851,41 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no DMARC p=reject record</t>
+          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Project Phoenix</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Team, only owner is disabled (Ben Okafor)</t>
+          <t>Doesn't receive mail but has no DMARC p=reject record</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B109" s="7" t="inlineStr">
@@ -4890,12 +4895,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Project Phoenix</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, no owner</t>
+          <t>Team, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
@@ -4912,34 +4917,34 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Provisioned</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
+          <t>Microsoft 365 group, no owner</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
+          <t>3 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>Provisioned</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>Excluded from "Require MFA for all users"</t>
+          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
         </is>
       </c>
     </row>
@@ -4951,17 +4956,17 @@
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>1 disabled account still licensed</t>
+          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>ben.okafor@fabrikam.example</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>Disabled, holding 1 licence</t>
+          <t>Excluded from "Require MFA for all users"</t>
         </is>
       </c>
     </row>
@@ -4973,17 +4978,17 @@
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including anonymous links</t>
+          <t>1 disabled account still licensed</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive</t>
+          <t>ben.okafor@fabrikam.example</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>Anyone links are allowed</t>
+          <t>Disabled, holding 1 licence</t>
         </is>
       </c>
     </row>
@@ -4995,29 +5000,24 @@
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>Anyone, including anonymous links</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Tenant SharePoint storage</t>
+          <t>SharePoint and OneDrive</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
-        </is>
-      </c>
-      <c r="E114" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone links are allowed</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
@@ -5027,12 +5027,12 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/finance</t>
+          <t>Tenant SharePoint storage</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
@@ -5054,12 +5054,12 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
+          <t>https://fabrikam.sharepoint.com/sites/finance</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
+          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
+          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
+          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -5108,12 +5108,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
+          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
+          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -5135,12 +5135,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/practice</t>
+          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
         </is>
       </c>
       <c r="E119" t="inlineStr">
@@ -5157,17 +5157,22 @@
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>1 app registration with expiring or expired credentials</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Old connector</t>
+          <t>https://fabrikam.sharepoint.com/sites/practice</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>The 1 credential expired, last on 1 Jan 2025</t>
+          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5179,17 +5184,17 @@
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>1 of 55 joined computers not in Intune</t>
+          <t>1 app registration with expiring or expired credentials</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>DESK-RECEPTION</t>
+          <t>Old connector</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>Hybrid joined, not managed by Intune</t>
+          <t>The 1 credential expired, last on 1 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -5201,17 +5206,17 @@
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 of 55 joined computers not in Intune</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>DESK-RECEPTION</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>Hybrid joined, not managed by Intune</t>
         </is>
       </c>
     </row>
@@ -5228,17 +5233,12 @@
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
           <t>Last check-in 38 days ago</t>
-        </is>
-      </c>
-      <c r="E123" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5255,12 +5255,17 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
           <t>Last check-in 38 days ago</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5277,7 +5282,7 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
@@ -5299,12 +5304,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 45 days ago</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -5316,17 +5321,17 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>1 of 57 device records unused for 90+ days</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>OLD-PC</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Windows, last seen 200 days ago</t>
+          <t>Last check-in 45 days ago</t>
         </is>
       </c>
     </row>
@@ -5338,17 +5343,17 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>1 domain with SPF problems</t>
+          <t>1 of 57 device records unused for 90+ days</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>OLD-PC</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
+          <t>Windows, last seen 200 days ago</t>
         </is>
       </c>
     </row>
@@ -5360,17 +5365,17 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
+          <t>1 domain with SPF problems</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
+          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
         </is>
       </c>
     </row>
@@ -5382,17 +5387,17 @@
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is on for the organisation</t>
+          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is allowed</t>
+          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
         </is>
       </c>
     </row>
@@ -5404,7 +5409,7 @@
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including guests, can invite guests</t>
+          <t>SMTP AUTH is on for the organisation</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
@@ -5414,7 +5419,7 @@
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>Guests can invite other guests</t>
+          <t>SMTP AUTH is allowed</t>
         </is>
       </c>
     </row>
@@ -5426,17 +5431,17 @@
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>Anyone, including guests, can invite guests</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>george.baker@fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>Guests can invite other guests</t>
         </is>
       </c>
     </row>
@@ -5453,17 +5458,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>owen.robinson@fabrikam.example</t>
+          <t>george.baker@fabrikam.example</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
           <t>Second factor is only Mobile phone (SMS or call)</t>
-        </is>
-      </c>
-      <c r="E133" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5480,12 +5480,17 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>owen.turner@fabrikam.example</t>
+          <t>owen.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
           <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5502,7 +5507,7 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>thomas.allen@fabrikam.example</t>
+          <t>owen.turner@fabrikam.example</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
@@ -5519,17 +5524,17 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>4 people can only use a text or call as a second factor</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Basic</t>
+          <t>thomas.allen@fabrikam.example</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
         </is>
       </c>
     </row>
@@ -5546,12 +5551,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Premium</t>
+          <t>Microsoft 365 Business Basic</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+          <t>2 of 13 unassigned, 9.80 GBP/month</t>
         </is>
       </c>
     </row>
@@ -5563,22 +5568,44 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Premium</t>
+        </is>
+      </c>
+      <c r="D138" s="7" t="inlineStr">
+        <is>
+          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B139" s="7" t="inlineStr">
+        <is>
           <t>Any user can register an app</t>
         </is>
       </c>
-      <c r="C138" t="inlineStr">
+      <c r="C139" t="inlineStr">
         <is>
           <t>Whole organisation</t>
         </is>
       </c>
-      <c r="D138" s="7" t="inlineStr">
+      <c r="D139" s="7" t="inlineStr">
         <is>
           <t>Users can register apps that nobody reviews</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E138"/>
+  <autoFilter ref="A1:E139"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -5752,7 +5779,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5784,7 +5811,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5799,7 +5826,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5814,7 +5841,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5829,7 +5856,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5844,7 +5871,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5859,7 +5886,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5874,7 +5901,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5889,7 +5916,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5904,7 +5931,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5919,7 +5946,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5934,7 +5961,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5949,7 +5976,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5964,7 +5991,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -5979,7 +6006,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87167824074</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -5994,7 +6021,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6009,7 +6036,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6024,7 +6051,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6039,7 +6066,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46304.99449074074</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6054,7 +6081,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6065,11 +6092,11 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Risky users</t>
+          <t>Mobile devices</t>
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6080,11 +6107,11 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Email domains</t>
+          <t>Automatic replies</t>
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6095,11 +6122,11 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Devices</t>
+          <t>Distribution lists</t>
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6110,11 +6137,11 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Directory sync</t>
+          <t>Risky users</t>
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6125,11 +6152,11 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive usage</t>
+          <t>Email domains</t>
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6140,11 +6167,11 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Shared files</t>
+          <t>Devices</t>
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6155,11 +6182,11 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SharePoint storage</t>
+          <t>Directory sync</t>
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46304.99450231482</v>
+        <v>46305.87168981481</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6170,20 +6197,110 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>SharePoint and OneDrive usage</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Shared files</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SharePoint storage</t>
+        </is>
+      </c>
+      <c r="B30" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
           <t>Microsoft 365 usage</t>
         </is>
       </c>
-      <c r="B28" s="12" t="n">
-        <v>46304.99450231482</v>
-      </c>
-      <c r="C28" t="inlineStr">
+      <c r="B31" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C31" t="inlineStr">
         <is>
           <t>Up to date</t>
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>App sign-ins</t>
+        </is>
+      </c>
+      <c r="B32" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Group nesting</t>
+        </is>
+      </c>
+      <c r="B33" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Departments and managers</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n">
+        <v>46305.87168981481</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C28"/>
+  <autoFilter ref="A1:C34"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Screenshots and examples for 2.2.0, on the README and the website
Every README image and example retaken from the demo, with the new pages (site and file permissions, mailbox, group and site pages, licence changes, mail flow, Teams, administrative units, the Evidence page, the Quarterly review design, roles and staff sign-in) shown in the README and on the website. The demo's site owners get their tenant's address.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -15,13 +15,13 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$55</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$62</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Checks'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$139</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$151</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Licences'!$A$1:$J$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Licences'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$34</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Data freshness'!$A$1:$C$39</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="4">'Data freshness'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +512,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 10 Oct 2026, 20:56 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 11 Oct 2026, 19:13 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -552,7 +552,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>33% on 12 Sep 2026</t>
+          <t>31% on 13 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -567,7 +567,7 @@
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>46.9% on 12 Sep 2026</t>
+          <t>47.8% on 13 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -582,7 +582,7 @@
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4 on 12 Sep 2026</t>
+          <t>4 on 13 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -597,7 +597,7 @@
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>52 on 12 Sep 2026</t>
+          <t>50 on 13 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -630,11 +630,11 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>35</v>
+        <v>40</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1 critical, 26 high, 53 medium, 58 low findings</t>
+          <t>1 critical, 28 high, 59 medium, 62 low findings</t>
         </is>
       </c>
     </row>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C14" s="7" t="n"/>
     </row>
@@ -685,7 +685,7 @@
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>54</v>
+        <v>61</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
         <is>
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="B19" s="9" t="n">
-        <v>138</v>
+        <v>150</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
@@ -730,7 +730,7 @@
         </is>
       </c>
       <c r="B21" s="9" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
@@ -764,7 +764,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:F55"/>
+  <dimension ref="A1:F62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -953,7 +953,7 @@
       </c>
       <c r="E6" s="7" t="inlineStr">
         <is>
-          <t>1 guest admin assignment</t>
+          <t>1 guest with admin roles</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
@@ -1236,7 +1236,7 @@
       </c>
       <c r="E15" s="7" t="inlineStr">
         <is>
-          <t>Outbound policies block automatic external forwarding</t>
+          <t>The default outbound policy blocks automatic external forwarding</t>
         </is>
       </c>
       <c r="F15" s="7" t="inlineStr">
@@ -1809,7 +1809,7 @@
       </c>
       <c r="F34" s="7" t="inlineStr">
         <is>
-          <t>Turn on DKIM for each domain in the Defender portal (Email authentication settings &gt; DKIM), publishing the two selector CNAME records it shows.</t>
+          <t>Turn on DKIM for each domain in the Defender portal (Email authentication settings &gt; DKIM), publishing the two selector CNAME records it shows. This applies to domains behind a mail gateway too when Microsoft 365 still sends for them (their SPF includes spf.protection.outlook.com); a gateway signs only the mail that goes out through it.</t>
         </is>
       </c>
     </row>
@@ -1836,7 +1836,7 @@
       </c>
       <c r="E35" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="F35" s="7" t="inlineStr">
@@ -1848,12 +1848,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Groups</t>
+          <t>Guests</t>
         </is>
       </c>
       <c r="B36" s="7" t="inlineStr">
         <is>
-          <t>Only chosen people can create teams and groups</t>
+          <t>No guest owns a team or group</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1863,12 +1863,12 @@
       </c>
       <c r="E36" s="7" t="inlineStr">
         <is>
-          <t>Only admins and members of Group creators can create teams and groups</t>
+          <t>No guest owns any of 9 teams and groups</t>
         </is>
       </c>
       <c r="F36" s="7" t="inlineStr">
         <is>
-          <t>Limit who can create teams and Microsoft 365 groups to a security group of people who will look after them (the Group.Unified directory setting, changed with Microsoft Graph PowerShell; needs Entra ID P1). Otherwise anyone can create a team, add guests to it and leave it behind.</t>
+          <t>Make a member of the organisation the owner of each listed team or group and remove the guest as owner (Teams admin center, or Microsoft 365 admin center &gt; Teams &amp; groups). An owner from outside can add members and guests, change settings and see everything in it, and nobody here is accountable for that.</t>
         </is>
       </c>
     </row>
@@ -1880,7 +1880,7 @@
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Unused groups and teams expire</t>
+          <t>Only chosen people can create teams and groups</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1890,44 +1890,39 @@
       </c>
       <c r="E37" s="7" t="inlineStr">
         <is>
-          <t>Unused teams and groups expire after 365 days</t>
+          <t>Only admins and members of Group creators can create teams and groups</t>
         </is>
       </c>
       <c r="F37" s="7" t="inlineStr">
         <is>
-          <t>Set a Microsoft 365 group expiration policy for all groups (Entra admin center &gt; Groups &gt; Expiration), for example 365 days. Groups in use renew automatically, owners are asked to renew the rest, and an expired group can be restored for 30 days. Needs Entra ID P1.</t>
+          <t>Limit who can create teams and Microsoft 365 groups to a security group of people who will look after them (the Group.Unified directory setting, changed with Microsoft Graph PowerShell; needs Entra ID P1). Otherwise anyone can create a team, add guests to it and leave it behind.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Devices</t>
+          <t>Groups</t>
         </is>
       </c>
       <c r="B38" s="7" t="inlineStr">
         <is>
-          <t>Managed devices meet compliance policies</t>
+          <t>Unused groups and teams expire</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Needs attention</t>
-        </is>
-      </c>
-      <c r="D38" t="inlineStr">
-        <is>
-          <t>Medium</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="E38" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>Unused teams and groups expire after 365 days</t>
         </is>
       </c>
       <c r="F38" s="7" t="inlineStr">
         <is>
-          <t>Open each non-compliant device in Intune (Devices &gt; Monitor &gt; Noncompliant devices) to see which setting fails, fix it or retire the device, and block non-compliant devices with a Conditional Access policy that requires a compliant device.</t>
+          <t>Set a Microsoft 365 group expiration policy for all groups (Entra admin center &gt; Groups &gt; Expiration), for example 365 days. Groups in use renew automatically, owners are asked to renew the rest, and an expired group can be restored for 30 days. Needs Entra ID P1.</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1934,7 @@
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Company computers are encrypted</t>
+          <t>Managed devices meet compliance policies</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1949,17 +1944,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E39" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 computers not encrypted</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="F39" s="7" t="inlineStr">
         <is>
-          <t>Turn on BitLocker (Windows) and FileVault (macOS) with an Intune disk encryption policy, with recovery keys escrowed to Entra ID, so a lost or stolen laptop doesn't expose the client's data.</t>
+          <t>Open each non-compliant device in Intune (Devices &gt; Monitor &gt; Noncompliant devices) to see which setting fails, fix it or retire the device, and block non-compliant devices with a Conditional Access policy that requires a compliant device.</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1966,7 @@
       </c>
       <c r="B40" s="7" t="inlineStr">
         <is>
-          <t>Windows computers still get security updates</t>
+          <t>Company computers are encrypted</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1986,12 +1981,12 @@
       </c>
       <c r="E40" s="7" t="inlineStr">
         <is>
-          <t>7 of 54 Windows computers past end of support</t>
+          <t>6 of 54 computers not encrypted</t>
         </is>
       </c>
       <c r="F40" s="7" t="inlineStr">
         <is>
-          <t>Upgrade computers on Windows 10 or an old Windows 11 release to the current Windows 11 release (Intune: Windows feature updates policy). Replace hardware that can't run Windows 11, or buy Extended Security Updates as a stopgap.</t>
+          <t>Turn on BitLocker (Windows) and FileVault (macOS) with an Intune disk encryption policy, with recovery keys escrowed to Entra ID, so a lost or stolen laptop doesn't expose the client's data.</t>
         </is>
       </c>
     </row>
@@ -2003,7 +1998,7 @@
       </c>
       <c r="B41" s="7" t="inlineStr">
         <is>
-          <t>Joined computers are managed by Intune</t>
+          <t>Windows computers still get security updates</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -2013,17 +2008,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
         <is>
-          <t>1 of 55 joined computers not in Intune</t>
+          <t>7 of 54 Windows computers past end of support</t>
         </is>
       </c>
       <c r="F41" s="7" t="inlineStr">
         <is>
-          <t>Enrol Entra-joined and hybrid-joined computers in Intune (automatic enrolment under Devices &gt; Enrollment &gt; Windows) so compliance, encryption and updates can be enforced on them.</t>
+          <t>Upgrade computers on Windows 10 or an old Windows 11 release to the current Windows 11 release (Intune: Windows feature updates policy). Replace hardware that can't run Windows 11, or buy Extended Security Updates as a stopgap.</t>
         </is>
       </c>
     </row>
@@ -2035,7 +2030,7 @@
       </c>
       <c r="B42" s="7" t="inlineStr">
         <is>
-          <t>Managed devices check in with Intune</t>
+          <t>Joined computers are managed by Intune</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -2050,12 +2045,12 @@
       </c>
       <c r="E42" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 of 55 joined computers not in Intune</t>
         </is>
       </c>
       <c r="F42" s="7" t="inlineStr">
         <is>
-          <t>Find out whether each device is lost, replaced or broken. Retire devices that are gone; for devices still in use, restart the Intune Management Extension or re-enrol.</t>
+          <t>Enrol Entra-joined and hybrid-joined computers in Intune (automatic enrolment under Devices &gt; Enrollment &gt; Windows) so compliance, encryption and updates can be enforced on them.</t>
         </is>
       </c>
     </row>
@@ -2067,7 +2062,7 @@
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>No old devices left in Entra ID</t>
+          <t>Managed devices check in with Intune</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -2082,39 +2077,44 @@
       </c>
       <c r="E43" s="7" t="inlineStr">
         <is>
-          <t>1 of 57 device records unused for 90+ days</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="F43" s="7" t="inlineStr">
         <is>
-          <t>Disable, then after 30 days delete, device records that haven't signed in for 90 days (Entra admin center &gt; Devices &gt; All devices, filter by activity). Old records can still hold BitLocker keys and count toward device limits.</t>
+          <t>Find out whether each device is lost, replaced or broken. Retire devices that are gone; for devices still in use, restart the Intune Management Extension or re-enrol.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Hybrid identity</t>
+          <t>Devices</t>
         </is>
       </c>
       <c r="B44" s="7" t="inlineStr">
         <is>
-          <t>Directory sync is running</t>
+          <t>No old devices left in Entra ID</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Not checked</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>Low</t>
         </is>
       </c>
       <c r="E44" s="7" t="inlineStr">
         <is>
-          <t>Cloud-only tenant: directory sync isn't turned on</t>
+          <t>1 of 57 device records unused for 90+ days</t>
         </is>
       </c>
       <c r="F44" s="7" t="inlineStr">
         <is>
-          <t>Check the Entra Connect server: that it is up, the Microsoft Azure AD Sync service is running and Synchronization Service Manager shows no errors. Until sync runs, accounts disabled or removed in Active Directory keep working in Microsoft 365. If the client has moved to cloud-only, turn directory sync off.</t>
+          <t>Disable, then after 30 days delete, device records that haven't signed in for 90 days (Entra admin center &gt; Devices &gt; All devices, filter by activity). Old records can still hold BitLocker keys and count toward device limits.</t>
         </is>
       </c>
     </row>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="B45" s="7" t="inlineStr">
         <is>
-          <t>Password hash sync is on</t>
+          <t>Directory sync is running</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -2141,7 +2141,7 @@
       </c>
       <c r="F45" s="7" t="inlineStr">
         <is>
-          <t>Turn on password hash synchronization in Entra Connect (Optional features), even when users sign in through federation or pass-through authentication. Entra ID can then detect leaked passwords, and sign-in can be switched to the cloud if the on-premises servers are down.</t>
+          <t>Check the Entra Connect server: that it is up, the Microsoft Azure AD Sync service is running and Synchronization Service Manager shows no errors. Until sync runs, accounts disabled or removed in Active Directory keep working in Microsoft 365. If the client has moved to cloud-only, turn directory sync off.</t>
         </is>
       </c>
     </row>
@@ -2153,66 +2153,61 @@
       </c>
       <c r="B46" s="7" t="inlineStr">
         <is>
-          <t>Admin accounts are cloud-only</t>
+          <t>Password hash sync is on</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Not checked</t>
         </is>
       </c>
       <c r="E46" s="7" t="inlineStr">
         <is>
-          <t>Cloud-only tenant: no accounts are synced from on-premises AD</t>
+          <t>Cloud-only tenant: directory sync isn't turned on</t>
         </is>
       </c>
       <c r="F46" s="7" t="inlineStr">
         <is>
-          <t>Give each admin a separate cloud-only account (for example on the .onmicrosoft.com domain) for their admin roles, and remove the roles from accounts synced from Active Directory. Otherwise anyone who takes over on-premises AD can reset those passwords and become an admin in Microsoft 365.</t>
+          <t>Turn on password hash synchronization in Entra Connect (Optional features), even when users sign in through federation or pass-through authentication. Entra ID can then detect leaked passwords, and sign-in can be switched to the cloud if the on-premises servers are down.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Hybrid identity</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
         <is>
-          <t>No unexpected changes to how domains sign in</t>
+          <t>Admin accounts are cloud-only</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Needs attention</t>
-        </is>
-      </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>High</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="E47" s="7" t="inlineStr">
         <is>
-          <t>1 domain had sign-in settings changed in the last 30 days</t>
+          <t>Cloud-only tenant: no accounts are synced from on-premises AD</t>
         </is>
       </c>
       <c r="F47" s="7" t="inlineStr">
         <is>
-          <t>Confirm with the client that each change was planned (for example, setting up AD FS or another identity provider). If it wasn't, an attacker with admin rights may have federated the domain to their own identity provider so they can sign in as any user without a password or MFA: switch the domain back to managed sign-in, remove unknown federation settings, reset admin credentials and review the audit log.</t>
+          <t>Give each admin a separate cloud-only account (for example on the .onmicrosoft.com domain) for their admin roles, and remove the roles from accounts synced from Active Directory. Otherwise anyone who takes over on-premises AD can reset those passwords and become an admin in Microsoft 365.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Sharing</t>
+          <t>Identity</t>
         </is>
       </c>
       <c r="B48" s="7" t="inlineStr">
         <is>
-          <t>No files are shared with anyone links</t>
+          <t>No unexpected changes to how domains sign in</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -2227,24 +2222,24 @@
       </c>
       <c r="E48" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>1 domain had sign-in settings changed in the last 30 days</t>
         </is>
       </c>
       <c r="F48" s="7" t="inlineStr">
         <is>
-          <t>Remove anyone links that are no longer needed, and set the rest to view-only with an expiry date. The Shared files report lists each one.</t>
+          <t>Confirm with the client that each change was planned (for example, setting up AD FS or another identity provider). If it wasn't, an attacker with admin rights may have federated the domain to their own identity provider so they can sign in as any user without a password or MFA: switch the domain back to managed sign-in, remove unknown federation settings, reset admin credentials and review the audit log.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Storage</t>
+          <t>Sharing</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>SharePoint storage isn't nearly full</t>
+          <t>No files are shared with anyone links</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2259,24 +2254,24 @@
       </c>
       <c r="E49" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="F49" s="7" t="inlineStr">
         <is>
-          <t>Free up space before the tenant runs out, when people can no longer save files. The SharePoint storage report shows where the space goes and what to clear first; otherwise buy Office 365 Extra File Storage.</t>
+          <t>Remove anyone links that are no longer needed, and set the rest to view-only with an expiry date. The Shared files report lists each one.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>Admins</t>
+          <t>Storage</t>
         </is>
       </c>
       <c r="B50" s="7" t="inlineStr">
         <is>
-          <t>Admins use phishing-resistant sign-in methods</t>
+          <t>SharePoint storage isn't nearly full</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2291,24 +2286,24 @@
       </c>
       <c r="E50" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="F50" s="7" t="inlineStr">
         <is>
-          <t>Have each listed admin register a passkey (in Microsoft Authenticator or on a security key) or Windows Hello for Business, then require the Phishing-resistant MFA authentication strength for admin roles in Conditional Access. Codes and push approvals can be relayed by a fake sign-in page; these can't.</t>
+          <t>Free up space before the tenant runs out, when people can no longer save files. The SharePoint storage report shows where the space goes and what to clear first; otherwise buy Office 365 Extra File Storage.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Sharing</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
         <is>
-          <t>Nobody relies on a text or call as their only second factor</t>
+          <t>Every site has at least two owners</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2318,98 +2313,113 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="E51" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="F51" s="7" t="inlineStr">
         <is>
-          <t>Ask these people to set up the Microsoft Authenticator app (the registration campaign in the authentication methods policy prompts them at sign-in), then turn off text message and voice call sign-in, or keep them only as a backup. Texts and calls can be intercepted or moved to an attacker's SIM.</t>
+          <t>Give each site a second owner (in the Microsoft 365 group, or as a site administrator) so access requests and content questions have someone to go to when one person leaves. The Site access report lists each site's owners.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Licences</t>
+          <t>Sharing</t>
         </is>
       </c>
       <c r="B52" s="7" t="inlineStr">
         <is>
-          <t>Every licence assignment works</t>
+          <t>Guests don't have full control of sites</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="E52" s="7" t="inlineStr">
         <is>
-          <t>Every licence assignment worked</t>
+          <t>1 guest with full control of 1 site</t>
         </is>
       </c>
       <c r="F52" s="7" t="inlineStr">
         <is>
-          <t>Fix each failed licence from the group's Licenses page in the Entra admin center: buy more licences when there aren't enough, remove licences that conflict, and correct usage locations. The Licences and subscriptions report explains each error.</t>
+          <t>Take guests out of each site's owners group and away from Full Control; give them Edit or Read through the site's members or visitors group instead. Full Control lets someone outside the organisation change who can open the site and delete anything on it. The Site permissions report lists them.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Licences</t>
+          <t>Sharing</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
         <is>
-          <t>No subscriptions are about to lapse</t>
+          <t>People outside can only view shared files</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E53" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions checked; none is lapsing</t>
+          <t>2 files and folders outside people can edit</t>
         </is>
       </c>
       <c r="F53" s="7" t="inlineStr">
         <is>
-          <t>Renew subscriptions in their grace period, buy or cancel trials people use before they end, and move people off suspended subscriptions. Billing &gt; Your products in the Microsoft 365 admin center (or Partner Center for subscriptions you sell) shows each one.</t>
+          <t>Change sharing with people outside the organisation to view-only unless they need to edit, and remove sharing that's no longer needed. The File and folder permissions report lists each person outside and what they can edit.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>Admins</t>
         </is>
       </c>
       <c r="B54" s="7" t="inlineStr">
         <is>
-          <t>No risky sign-ins succeeded</t>
+          <t>Admins use phishing-resistant sign-in methods</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Not checked</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E54" s="7" t="inlineStr">
         <is>
-          <t>Sign-in risk needs Entra ID P2</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="F54" s="7" t="inlineStr">
         <is>
-          <t>Check each sign-in with the person. If they don't recognise it, reset their password, sign them out everywhere (revoke sessions), and check their MFA methods, inbox rules and app consents; then confirm the account compromised in Entra ID Protection. Add a Conditional Access policy that asks for MFA on medium and high sign-in risk. The Sign-in activity report lists every risky sign-in.</t>
+          <t>Have each listed admin register a passkey (in Microsoft Authenticator or on a security key) or Windows Hello for Business, then require the Phishing-resistant MFA authentication strength for admin roles in Conditional Access. Codes and push approvals can be relayed by a fake sign-in page; these can't.</t>
         </is>
       </c>
     </row>
@@ -2421,27 +2431,231 @@
       </c>
       <c r="B55" s="7" t="inlineStr">
         <is>
+          <t>Nobody relies on a text or call as their only second factor</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>Ask these people to set up the Microsoft Authenticator app (the registration campaign in the authentication methods policy prompts them at sign-in), then turn off text message and voice call sign-in, or keep them only as a backup. Texts and calls can be intercepted or moved to an attacker's SIM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Licences</t>
+        </is>
+      </c>
+      <c r="B56" s="7" t="inlineStr">
+        <is>
+          <t>Every licence assignment works</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E56" s="7" t="inlineStr">
+        <is>
+          <t>Every licence assignment worked</t>
+        </is>
+      </c>
+      <c r="F56" s="7" t="inlineStr">
+        <is>
+          <t>Fix each failed licence from the group's Licenses page in the Entra admin center: buy more licences when there aren't enough, remove licences that conflict, and correct usage locations. The Licences and subscriptions report explains each error.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Licences</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>No subscriptions are about to lapse</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>2 subscriptions checked; none is lapsing</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>Renew subscriptions in their grace period, buy or cancel trials people use before they end, and move people off suspended subscriptions. Billing &gt; Your products in the Microsoft 365 admin center (or Partner Center for subscriptions you sell) shows each one.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B58" s="7" t="inlineStr">
+        <is>
+          <t>No risky sign-ins succeeded</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Not checked</t>
+        </is>
+      </c>
+      <c r="E58" s="7" t="inlineStr">
+        <is>
+          <t>Sign-in risk needs Entra ID P2</t>
+        </is>
+      </c>
+      <c r="F58" s="7" t="inlineStr">
+        <is>
+          <t>Check each sign-in with the person. If they don't recognise it, reset their password, sign them out everywhere (revoke sessions), and check their MFA methods, inbox rules and app consents; then confirm the account compromised in Entra ID Protection. Add a Conditional Access policy that asks for MFA on medium and high sign-in risk. The Sign-in activity report lists every risky sign-in.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
           <t>No accounts are at risk in Entra ID Protection</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
+      <c r="C59" t="inlineStr">
         <is>
           <t>Not checked</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E59" s="7" t="inlineStr">
         <is>
           <t>Risky users need Entra ID P2</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
+      <c r="F59" s="7" t="inlineStr">
         <is>
           <t>Check each account with the person. If they don't recognise recent sign-ins, reset the password, sign them out everywhere (revoke sessions), and check their MFA methods, inbox rules and app consents; then confirm the account compromised or dismiss the risk in Entra ID Protection. Add a Conditional Access policy that asks for a secure password change on high user risk. The Risky users report lists each account.</t>
         </is>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>Accounts</t>
+        </is>
+      </c>
+      <c r="B60" s="7" t="inlineStr">
+        <is>
+          <t>No account reports to a blocked manager</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="E60" s="7" t="inlineStr">
+        <is>
+          <t>1 account reports to a blocked manager</t>
+        </is>
+      </c>
+      <c r="F60" s="7" t="inlineStr">
+        <is>
+          <t>Set a current manager on each listed account (Entra admin center &gt; Users &gt; Properties &gt; Manager, or in on-premises AD for synced accounts). The manager is where approvals, leaver notices and access reviews go; when they've left, those go nowhere, and their blocked account is usually waiting to be deleted too.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>No mailbox is nearly full</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="E61" s="7" t="inlineStr">
+        <is>
+          <t>3 mailboxes at or over 90% of quota</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr">
+        <is>
+          <t>Turn on the online archive for each listed mailbox (Exchange admin center &gt; Mailboxes &gt; Manage mailbox archive) with a retention policy that moves old mail into it, or clear large old items. A mailbox at its quota can't send, and soon after can't receive.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>Storage</t>
+        </is>
+      </c>
+      <c r="B62" s="7" t="inlineStr">
+        <is>
+          <t>No OneDrive is nearly full</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="E62" s="7" t="inlineStr">
+        <is>
+          <t>None of 54 OneDrives is over 90% of its quota</t>
+        </is>
+      </c>
+      <c r="F62" s="7" t="inlineStr">
+        <is>
+          <t>Ask each listed person to clear or archive old files, or raise their OneDrive quota (SharePoint admin center &gt; Settings &gt; OneDrive Storage limit, up to 5 TB with a qualifying licence). A full OneDrive stops syncing and saving.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F55"/>
+  <autoFilter ref="A1:F62"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -2461,7 +2675,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E139"/>
+  <dimension ref="A1:E151"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -2572,7 +2786,7 @@
       </c>
       <c r="B5" s="7" t="inlineStr">
         <is>
-          <t>1 guest admin assignment</t>
+          <t>1 guest with admin roles</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -4323,7 +4537,7 @@
       </c>
       <c r="D83" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 8 Oct 2026</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 9 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4335,105 +4549,105 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Clients (Finance / Documents)</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
         <is>
-          <t>Anyone can edit, link never expires</t>
+          <t>No enabled owner (Microsoft 365 group)</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
+          <t>Old Projects</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>Anyone can view</t>
+          <t>No enabled owner (site administrators)</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>Practice Management</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 21 Apr 2026</t>
+          <t>One owner (Microsoft 365 group)</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>Staff Intranet</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 5 Mar 2026</t>
+          <t>One owner (site administrators)</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B88" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>1 guest with full control of 1 site</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>accounts@hollis-partners.example on Finance</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 2 Jun 2026</t>
+          <t>Full Control, given Full Control directly</t>
         </is>
       </c>
     </row>
@@ -4450,12 +4664,12 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 5 Feb 2026</t>
+          <t>Licensed member, last signed in 22 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -4472,12 +4686,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 3 Jun 2026</t>
+          <t>Licensed member, last signed in 6 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -4494,19 +4708,19 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 7 Jul 2026</t>
+          <t>Licensed member, last signed in 3 Jun 2026</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B92" s="7" t="inlineStr">
@@ -4516,12 +4730,12 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Guest, never signed in, created ?</t>
+          <t>Licensed member, last signed in 6 Feb 2026</t>
         </is>
       </c>
     </row>
@@ -4533,17 +4747,17 @@
       </c>
       <c r="B93" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>7 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with Authenticator app</t>
+          <t>Licensed member, last signed in 4 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -4555,39 +4769,39 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>7 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with no MFA method at all</t>
+          <t>Licensed member, last signed in 8 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>1 app with privileged roles</t>
+          <t>7 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Some app</t>
+          <t>g#EXT#@fabrikam.example</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>App holding Exchange Administrator</t>
+          <t>Guest, never signed in, created ?</t>
         </is>
       </c>
     </row>
@@ -4599,17 +4813,17 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>Users can consent to any app</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Any user can grant any app access to their mail and files</t>
+          <t>Global Administrator; signs in with Authenticator app</t>
         </is>
       </c>
     </row>
@@ -4621,17 +4835,17 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>Global Administrator; signs in with no MFA method at all</t>
         </is>
       </c>
     </row>
@@ -4643,17 +4857,17 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>1 app with privileged roles</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>Some app</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>App holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -4665,22 +4879,17 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>Users can consent to any app</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
-        </is>
-      </c>
-      <c r="E99" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Any user can grant any app access to their mail and files</t>
         </is>
       </c>
     </row>
@@ -4697,7 +4906,7 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
@@ -4719,7 +4928,7 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
@@ -4741,12 +4950,17 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -4763,7 +4977,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
@@ -4785,7 +4999,7 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
@@ -4807,7 +5021,7 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
@@ -4824,17 +5038,17 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>1 mail domain without DKIM</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -4846,39 +5060,39 @@
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B108" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no DMARC p=reject record</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -4890,39 +5104,39 @@
       </c>
       <c r="B109" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>1 mail domain without DKIM</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Project Phoenix</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
         <is>
-          <t>Team, only owner is disabled (Ben Okafor)</t>
+          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B110" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, no owner</t>
+          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
         </is>
       </c>
     </row>
@@ -4934,17 +5148,17 @@
       </c>
       <c r="B111" s="7" t="inlineStr">
         <is>
-          <t>3 teams and groups without an owner</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Provisioned</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
+          <t>Doesn't receive mail but has no DMARC p=reject record</t>
         </is>
       </c>
     </row>
@@ -4956,311 +5170,286 @@
       </c>
       <c r="B112" s="7" t="inlineStr">
         <is>
-          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>Project Phoenix</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
         <is>
-          <t>Excluded from "Require MFA for all users"</t>
+          <t>Team, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B113" s="7" t="inlineStr">
         <is>
-          <t>1 disabled account still licensed</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>ben.okafor@fabrikam.example</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
         <is>
-          <t>Disabled, holding 1 licence</t>
+          <t>Microsoft 365 group, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B114" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including anonymous links</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
         <is>
-          <t>Anyone links are allowed</t>
+          <t>Microsoft 365 group, no owner</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Tenant SharePoint storage</t>
+          <t>Provisioned</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
-        </is>
-      </c>
-      <c r="E115" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>Enforced by Require MFA for all users, with 1 exclusion to review</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/finance</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
-        </is>
-      </c>
-      <c r="E116" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Excluded from "Require MFA for all users"</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B117" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>1 disabled account still licensed</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
+          <t>ben.okafor@fabrikam.example</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
         <is>
-          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
-        </is>
-      </c>
-      <c r="E117" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Disabled, holding 1 licence</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B118" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>Anyone, including anonymous links</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
+          <t>SharePoint and OneDrive</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
         <is>
-          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
-        </is>
-      </c>
-      <c r="E118" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone links are allowed</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B119" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
+          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
         <is>
-          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
-        </is>
-      </c>
-      <c r="E119" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone can view</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B120" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/practice</t>
+          <t>Open day flyer.pdf (Marketing / Documents)</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
         <is>
-          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
-        </is>
-      </c>
-      <c r="E120" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone can view, link never expires</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B121" s="7" t="inlineStr">
         <is>
-          <t>1 app registration with expiring or expired credentials</t>
+          <t>2 files and folders outside people can edit</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Old connector</t>
+          <t>Budget.xlsx (Finance / Documents)</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
         <is>
-          <t>The 1 credential expired, last on 1 Jan 2025</t>
+          <t>Can be edited by accountant@hargreaves-partners.example</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>1 of 55 joined computers not in Intune</t>
+          <t>2 files and folders outside people can edit</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>DESK-RECEPTION</t>
+          <t>Lab dockets (Patient Records / Documents)</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Hybrid joined, not managed by Intune</t>
+          <t>Can be edited by orders@dentallab.example</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B123" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>accounts@fabrikam.example</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>44.8 GB of 49.5 GB (91%), no archive</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>47.2 GB of 49.5 GB (95%), no archive</t>
         </is>
       </c>
       <c r="E124" t="inlineStr">
@@ -5272,44 +5461,54 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B125" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>thomas.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>45.6 GB of 49.5 GB (92%), no archive</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>Tenant SharePoint storage</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5321,17 +5520,22 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>https://fabrikam.sharepoint.com/sites/finance</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 45 days ago</t>
+          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5343,17 +5547,22 @@
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>1 of 57 device records unused for 90+ days</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>OLD-PC</t>
+          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Windows, last seen 200 days ago</t>
+          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5365,17 +5574,22 @@
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>1 domain with SPF problems</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
+          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5387,17 +5601,22 @@
       </c>
       <c r="B130" s="7" t="inlineStr">
         <is>
-          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
+          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5409,17 +5628,22 @@
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is on for the organisation</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>https://fabrikam.sharepoint.com/sites/practice</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is allowed</t>
+          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5431,17 +5655,17 @@
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including guests, can invite guests</t>
+          <t>1 account reports to a blocked manager</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Guests can invite other guests</t>
+          <t>Reports to Ben Okafor, whose sign-in is blocked</t>
         </is>
       </c>
     </row>
@@ -5453,17 +5677,17 @@
       </c>
       <c r="B133" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>1 app registration with expiring or expired credentials</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>george.baker@fabrikam.example</t>
+          <t>Old connector</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>The 1 credential expired, last on 1 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -5475,22 +5699,17 @@
       </c>
       <c r="B134" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>1 of 55 joined computers not in Intune</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>owen.robinson@fabrikam.example</t>
+          <t>DESK-RECEPTION</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
-        </is>
-      </c>
-      <c r="E134" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Hybrid joined, not managed by Intune</t>
         </is>
       </c>
     </row>
@@ -5502,17 +5721,17 @@
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>owen.turner@fabrikam.example</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -5524,17 +5743,22 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>thomas.allen@fabrikam.example</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>Last check-in 38 days ago</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5546,17 +5770,17 @@
       </c>
       <c r="B137" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Basic</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -5568,17 +5792,17 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Premium</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -5590,22 +5814,291 @@
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
+          <t>5 devices haven't checked in for 30+ days</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+        </is>
+      </c>
+      <c r="D139" s="7" t="inlineStr">
+        <is>
+          <t>Last check-in 45 days ago</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B140" s="7" t="inlineStr">
+        <is>
+          <t>1 of 57 device records unused for 90+ days</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>OLD-PC</t>
+        </is>
+      </c>
+      <c r="D140" s="7" t="inlineStr">
+        <is>
+          <t>Windows, last seen 200 days ago</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B141" s="7" t="inlineStr">
+        <is>
+          <t>1 domain with SPF problems</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>parked.example</t>
+        </is>
+      </c>
+      <c r="D141" s="7" t="inlineStr">
+        <is>
+          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B142" s="7" t="inlineStr">
+        <is>
+          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D142" s="7" t="inlineStr">
+        <is>
+          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B143" s="7" t="inlineStr">
+        <is>
+          <t>SMTP AUTH is on for the organisation</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>Whole organisation</t>
+        </is>
+      </c>
+      <c r="D143" s="7" t="inlineStr">
+        <is>
+          <t>SMTP AUTH is allowed</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B144" s="7" t="inlineStr">
+        <is>
+          <t>Anyone, including guests, can invite guests</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>Whole organisation</t>
+        </is>
+      </c>
+      <c r="D144" s="7" t="inlineStr">
+        <is>
+          <t>Guests can invite other guests</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B145" s="7" t="inlineStr">
+        <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>george.baker@fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D145" s="7" t="inlineStr">
+        <is>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B146" s="7" t="inlineStr">
+        <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>owen.robinson@fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D146" s="7" t="inlineStr">
+        <is>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B147" s="7" t="inlineStr">
+        <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>owen.turner@fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D147" s="7" t="inlineStr">
+        <is>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B148" s="7" t="inlineStr">
+        <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>thomas.allen@fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D148" s="7" t="inlineStr">
+        <is>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B149" s="7" t="inlineStr">
+        <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Basic</t>
+        </is>
+      </c>
+      <c r="D149" s="7" t="inlineStr">
+        <is>
+          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B150" s="7" t="inlineStr">
+        <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Premium</t>
+        </is>
+      </c>
+      <c r="D150" s="7" t="inlineStr">
+        <is>
+          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B151" s="7" t="inlineStr">
+        <is>
           <t>Any user can register an app</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
+      <c r="C151" t="inlineStr">
         <is>
           <t>Whole organisation</t>
         </is>
       </c>
-      <c r="D139" s="7" t="inlineStr">
+      <c r="D151" s="7" t="inlineStr">
         <is>
           <t>Users can register apps that nobody reviews</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E139"/>
+  <autoFilter ref="A1:E151"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -5779,7 +6272,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="31" customWidth="1" min="1" max="1"/>
@@ -5811,7 +6304,7 @@
         </is>
       </c>
       <c r="B2" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -5826,7 +6319,7 @@
         </is>
       </c>
       <c r="B3" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -5841,7 +6334,7 @@
         </is>
       </c>
       <c r="B4" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -5856,7 +6349,7 @@
         </is>
       </c>
       <c r="B5" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -5871,7 +6364,7 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -5886,7 +6379,7 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -5901,7 +6394,7 @@
         </is>
       </c>
       <c r="B8" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5916,7 +6409,7 @@
         </is>
       </c>
       <c r="B9" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -5931,7 +6424,7 @@
         </is>
       </c>
       <c r="B10" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -5946,7 +6439,7 @@
         </is>
       </c>
       <c r="B11" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -5961,7 +6454,7 @@
         </is>
       </c>
       <c r="B12" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -5976,7 +6469,7 @@
         </is>
       </c>
       <c r="B13" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -5991,7 +6484,7 @@
         </is>
       </c>
       <c r="B14" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -6006,7 +6499,7 @@
         </is>
       </c>
       <c r="B15" s="12" t="n">
-        <v>46305.87167824074</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -6021,7 +6514,7 @@
         </is>
       </c>
       <c r="B16" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -6036,7 +6529,7 @@
         </is>
       </c>
       <c r="B17" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -6051,7 +6544,7 @@
         </is>
       </c>
       <c r="B18" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -6066,7 +6559,7 @@
         </is>
       </c>
       <c r="B19" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -6081,7 +6574,7 @@
         </is>
       </c>
       <c r="B20" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.80025462963</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -6096,7 +6589,7 @@
         </is>
       </c>
       <c r="B21" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -6111,7 +6604,7 @@
         </is>
       </c>
       <c r="B22" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -6126,7 +6619,7 @@
         </is>
       </c>
       <c r="B23" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -6141,7 +6634,7 @@
         </is>
       </c>
       <c r="B24" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -6156,7 +6649,7 @@
         </is>
       </c>
       <c r="B25" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -6171,7 +6664,7 @@
         </is>
       </c>
       <c r="B26" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -6186,7 +6679,7 @@
         </is>
       </c>
       <c r="B27" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -6201,7 +6694,7 @@
         </is>
       </c>
       <c r="B28" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -6216,7 +6709,7 @@
         </is>
       </c>
       <c r="B29" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -6231,7 +6724,7 @@
         </is>
       </c>
       <c r="B30" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -6242,11 +6735,11 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Microsoft 365 usage</t>
+          <t>Site access</t>
         </is>
       </c>
       <c r="B31" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -6257,11 +6750,11 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>App sign-ins</t>
+          <t>Site permissions</t>
         </is>
       </c>
       <c r="B32" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -6272,11 +6765,11 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Group nesting</t>
+          <t>Microsoft 365 usage</t>
         </is>
       </c>
       <c r="B33" s="12" t="n">
-        <v>46305.87168981481</v>
+        <v>46306.8002662037</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -6287,20 +6780,95 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>Teams</t>
+        </is>
+      </c>
+      <c r="B34" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Mail flow</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>App sign-ins</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Group nesting</t>
+        </is>
+      </c>
+      <c r="B37" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
           <t>Departments and managers</t>
         </is>
       </c>
-      <c r="B34" s="12" t="n">
-        <v>46305.87168981481</v>
-      </c>
-      <c r="C34" t="inlineStr">
+      <c r="B38" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C38" t="inlineStr">
         <is>
           <t>Up to date</t>
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Administrative units</t>
+        </is>
+      </c>
+      <c r="B39" s="12" t="n">
+        <v>46306.8002662037</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Up to date</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:C34"/>
+  <autoFilter ref="A1:C39"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>

</xml_diff>

<commit_message>
Make Ink the default colour, with a redrawn mark
The 2.4.0 bottle green filled the menu and every link, so busy pages like
Today were hard to focus on. Ink is plain grey paper, a light menu and one
blue-black accent (#2b4a6b, #9fb8d4 at night), leaving colour for severity
and status.

- tokens.css and themes.css: Ink is the default theme; bottle green moves
  to its own "bottle" key on the Account page. A stored "green" (the column
  default and 2.4.0's default) reads as the new default, so other saved
  choices are kept.
- Reports and emails for an MSP without a brand colour, and the demo MSP,
  use the ink.
- The mark: a solid white shield with its tick cut out, on a flat ink tile,
  in the menu, the favicons, the website and its social card.
- Website, README badges, DESIGN.md and the screenshots and example
  reports follow.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -49,7 +49,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000D7A5F"/>
+      <color rgb="002B4A6B"/>
       <sz val="16"/>
     </font>
     <font>
@@ -77,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D7A5F"/>
+        <fgColor rgb="002B4A6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +91,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="000D7A5F"/>
+        <color rgb="002B4A6B"/>
       </bottom>
     </border>
   </borders>
@@ -515,7 +515,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 16 Oct 2026, 11:17 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 16 Oct 2026, 12:33 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 13 Oct 2026</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 14 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -7094,7 +7094,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -7124,7 +7124,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -7139,7 +7139,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -7154,7 +7154,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -7169,7 +7169,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -7184,7 +7184,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -7199,7 +7199,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -7214,7 +7214,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -7244,7 +7244,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -7259,7 +7259,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -7289,7 +7289,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -7304,7 +7304,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -7349,7 +7349,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -7364,7 +7364,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -7409,7 +7409,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -7454,7 +7454,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -7484,7 +7484,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -7499,7 +7499,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -7514,7 +7514,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7529,7 +7529,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -7544,7 +7544,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -7559,7 +7559,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -7604,7 +7604,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -7619,7 +7619,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -7634,7 +7634,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -7649,7 +7649,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -7664,7 +7664,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -7679,7 +7679,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -7694,7 +7694,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -7709,7 +7709,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Make Ink the default colour, with a redrawn mark (#173)
Ink becomes the default for the portal, demo, website and reports without a brand colour; bottle green and the others stay in Appearance, and the mark is redrawn.
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -49,7 +49,7 @@
     </font>
     <font>
       <b val="1"/>
-      <color rgb="000D7A5F"/>
+      <color rgb="002B4A6B"/>
       <sz val="16"/>
     </font>
     <font>
@@ -77,7 +77,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000D7A5F"/>
+        <fgColor rgb="002B4A6B"/>
       </patternFill>
     </fill>
   </fills>
@@ -91,7 +91,7 @@
     </border>
     <border>
       <bottom style="thin">
-        <color rgb="000D7A5F"/>
+        <color rgb="002B4A6B"/>
       </bottom>
     </border>
   </borders>
@@ -515,7 +515,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 16 Oct 2026, 11:17 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 16 Oct 2026, 12:33 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 13 Oct 2026</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 14 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
         </is>
       </c>
       <c r="B2" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -7094,7 +7094,7 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -7109,7 +7109,7 @@
         </is>
       </c>
       <c r="B4" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -7124,7 +7124,7 @@
         </is>
       </c>
       <c r="B5" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -7139,7 +7139,7 @@
         </is>
       </c>
       <c r="B6" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -7154,7 +7154,7 @@
         </is>
       </c>
       <c r="B7" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -7169,7 +7169,7 @@
         </is>
       </c>
       <c r="B8" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -7184,7 +7184,7 @@
         </is>
       </c>
       <c r="B9" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -7199,7 +7199,7 @@
         </is>
       </c>
       <c r="B10" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -7214,7 +7214,7 @@
         </is>
       </c>
       <c r="B11" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -7229,7 +7229,7 @@
         </is>
       </c>
       <c r="B12" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -7244,7 +7244,7 @@
         </is>
       </c>
       <c r="B13" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -7259,7 +7259,7 @@
         </is>
       </c>
       <c r="B14" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -7274,7 +7274,7 @@
         </is>
       </c>
       <c r="B15" s="13" t="n">
-        <v>46311.46931712963</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -7289,7 +7289,7 @@
         </is>
       </c>
       <c r="B16" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52193287037</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -7304,7 +7304,7 @@
         </is>
       </c>
       <c r="B17" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -7319,7 +7319,7 @@
         </is>
       </c>
       <c r="B18" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -7334,7 +7334,7 @@
         </is>
       </c>
       <c r="B19" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -7349,7 +7349,7 @@
         </is>
       </c>
       <c r="B20" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -7364,7 +7364,7 @@
         </is>
       </c>
       <c r="B21" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -7379,7 +7379,7 @@
         </is>
       </c>
       <c r="B22" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -7394,7 +7394,7 @@
         </is>
       </c>
       <c r="B23" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -7409,7 +7409,7 @@
         </is>
       </c>
       <c r="B24" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -7424,7 +7424,7 @@
         </is>
       </c>
       <c r="B25" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -7439,7 +7439,7 @@
         </is>
       </c>
       <c r="B26" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -7454,7 +7454,7 @@
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -7469,7 +7469,7 @@
         </is>
       </c>
       <c r="B28" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -7484,7 +7484,7 @@
         </is>
       </c>
       <c r="B29" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -7499,7 +7499,7 @@
         </is>
       </c>
       <c r="B30" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -7514,7 +7514,7 @@
         </is>
       </c>
       <c r="B31" s="13" t="n">
-        <v>46311.4693287037</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7529,7 +7529,7 @@
         </is>
       </c>
       <c r="B32" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -7544,7 +7544,7 @@
         </is>
       </c>
       <c r="B33" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -7559,7 +7559,7 @@
         </is>
       </c>
       <c r="B34" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -7574,7 +7574,7 @@
         </is>
       </c>
       <c r="B35" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -7589,7 +7589,7 @@
         </is>
       </c>
       <c r="B36" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52194444444</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -7604,7 +7604,7 @@
         </is>
       </c>
       <c r="B37" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -7619,7 +7619,7 @@
         </is>
       </c>
       <c r="B38" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -7634,7 +7634,7 @@
         </is>
       </c>
       <c r="B39" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -7649,7 +7649,7 @@
         </is>
       </c>
       <c r="B40" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -7664,7 +7664,7 @@
         </is>
       </c>
       <c r="B41" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -7679,7 +7679,7 @@
         </is>
       </c>
       <c r="B42" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -7694,7 +7694,7 @@
         </is>
       </c>
       <c r="B43" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -7709,7 +7709,7 @@
         </is>
       </c>
       <c r="B44" s="13" t="n">
-        <v>46311.46934027778</v>
+        <v>46311.52195601852</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Retake the screenshots and example reports for 2.5.0
</commit_message>
<xml_diff>
--- a/examples/monthly-security-licensing-review.xlsx
+++ b/examples/monthly-security-licensing-review.xlsx
@@ -17,7 +17,7 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'Summary'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Checks'!$A$1:$F$72</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'Checks'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$172</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Findings'!$A$1:$E$175</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'Findings'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Licences'!$A$1:$J$3</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="3">'Licences'!$1:$1</definedName>
@@ -30,10 +30,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="d mmm yyyy hh:mm"/>
-    <numFmt numFmtId="166" formatCode="0.0%"/>
   </numFmts>
   <fonts count="7">
     <font>
@@ -98,7 +97,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -112,9 +111,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left"/>
@@ -515,7 +511,7 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Prepared by Harbour IT · 16 Oct 2026, 13:36 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
+          <t>Prepared by Harbour IT · 17 Oct 2026, 10:10 UTC · Microsoft 365 tenant fabrikam.onmicrosoft.com</t>
         </is>
       </c>
     </row>
@@ -555,7 +551,7 @@
       </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
-          <t>32% on 18 Sep 2026</t>
+          <t>32% on 19 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -565,12 +561,12 @@
           <t>Users with MFA</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>0.509</v>
+      <c r="B8" s="6" t="n">
+        <v>0.5</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>45.6% on 18 Sep 2026</t>
+          <t>44.7% on 19 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -580,12 +576,12 @@
           <t>Privileged accounts</t>
         </is>
       </c>
-      <c r="B9" s="9" t="n">
+      <c r="B9" s="8" t="n">
         <v>4</v>
       </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
-          <t>4 on 18 Sep 2026</t>
+          <t>4 on 19 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -595,12 +591,12 @@
           <t>Licensed users</t>
         </is>
       </c>
-      <c r="B10" s="9" t="n">
+      <c r="B10" s="8" t="n">
         <v>54</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>51 on 18 Sep 2026</t>
+          <t>51 on 19 Sep 2026</t>
         </is>
       </c>
     </row>
@@ -610,8 +606,8 @@
           <t>Inactive accounts</t>
         </is>
       </c>
-      <c r="B11" s="10" t="n">
-        <v>7</v>
+      <c r="B11" s="9" t="n">
+        <v>8</v>
       </c>
       <c r="C11" s="7" t="n"/>
     </row>
@@ -621,7 +617,7 @@
           <t>Licence waste / month (GBP)</t>
         </is>
       </c>
-      <c r="B12" s="9" t="n">
+      <c r="B12" s="8" t="n">
         <v>164.4</v>
       </c>
       <c r="C12" s="7" t="n"/>
@@ -632,12 +628,12 @@
           <t>Checks needing attention</t>
         </is>
       </c>
-      <c r="B13" s="10" t="n">
-        <v>48</v>
+      <c r="B13" s="9" t="n">
+        <v>49</v>
       </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
-          <t>1 critical, 31 high, 99 medium, 40 low findings</t>
+          <t>1 critical, 31 high, 101 medium, 41 low findings</t>
         </is>
       </c>
     </row>
@@ -647,8 +643,8 @@
           <t>Checks passed</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n">
-        <v>16</v>
+      <c r="B14" s="9" t="n">
+        <v>15</v>
       </c>
       <c r="C14" s="7" t="n"/>
     </row>
@@ -658,7 +654,7 @@
           <t>Not checked</t>
         </is>
       </c>
-      <c r="B15" s="10" t="n">
+      <c r="B15" s="9" t="n">
         <v>7</v>
       </c>
       <c r="C15" s="7" t="n"/>
@@ -682,12 +678,12 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="10" t="inlineStr">
         <is>
           <t>Checks</t>
         </is>
       </c>
-      <c r="B18" s="10" t="n">
+      <c r="B18" s="9" t="n">
         <v>71</v>
       </c>
       <c r="C18" s="7" t="inlineStr">
@@ -697,13 +693,13 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="10" t="inlineStr">
         <is>
           <t>Findings</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
-        <v>171</v>
+      <c r="B19" s="9" t="n">
+        <v>174</v>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
@@ -712,12 +708,12 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Licences</t>
         </is>
       </c>
-      <c r="B20" s="10" t="n">
+      <c r="B20" s="9" t="n">
         <v>2</v>
       </c>
       <c r="C20" s="7" t="inlineStr">
@@ -727,12 +723,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="10" t="inlineStr">
         <is>
           <t>Data freshness</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="9" t="n">
         <v>43</v>
       </c>
       <c r="C21" s="7" t="inlineStr">
@@ -1020,7 +1016,7 @@
       </c>
       <c r="E8" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
@@ -1052,7 +1048,7 @@
       </c>
       <c r="E9" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -1084,7 +1080,7 @@
       </c>
       <c r="E10" s="7" t="inlineStr">
         <is>
-          <t>1 disabled account still licensed</t>
+          <t>1 disabled account still licensed (not counting 1 shared mailbox that needs one)</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
@@ -1261,12 +1257,17 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Needs attention</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E16" s="7" t="inlineStr">
         <is>
-          <t>All 3 shared mailboxes block sign-in</t>
+          <t>1 of 3 shared mailboxes allows sign-in</t>
         </is>
       </c>
       <c r="F16" s="7" t="inlineStr">
@@ -2988,7 +2989,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E172"/>
+  <dimension ref="A1:E175"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -3082,7 +3083,7 @@
       </c>
       <c r="C4" s="7" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>sam.carter_consultants.example#EXT#@fabrikam.onmicrosoft.com</t>
         </is>
       </c>
       <c r="D4" s="7" t="inlineStr">
@@ -3126,7 +3127,7 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>sam.carter_consultants.example#EXT#@fabrikam.onmicrosoft.com</t>
         </is>
       </c>
       <c r="D6" s="7" t="inlineStr">
@@ -4290,7 +4291,7 @@
       </c>
       <c r="B58" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C58" s="7" t="inlineStr">
@@ -4312,7 +4313,7 @@
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
@@ -4334,7 +4335,7 @@
       </c>
       <c r="B60" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C60" s="7" t="inlineStr">
@@ -4356,7 +4357,7 @@
       </c>
       <c r="B61" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C61" s="7" t="inlineStr">
@@ -4378,7 +4379,7 @@
       </c>
       <c r="B62" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C62" s="7" t="inlineStr">
@@ -4400,7 +4401,7 @@
       </c>
       <c r="B63" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C63" s="7" t="inlineStr">
@@ -4422,7 +4423,7 @@
       </c>
       <c r="B64" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C64" s="7" t="inlineStr">
@@ -4444,7 +4445,7 @@
       </c>
       <c r="B65" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C65" s="7" t="inlineStr">
@@ -4466,7 +4467,7 @@
       </c>
       <c r="B66" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C66" s="7" t="inlineStr">
@@ -4488,7 +4489,7 @@
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
@@ -4510,7 +4511,7 @@
       </c>
       <c r="B68" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C68" s="7" t="inlineStr">
@@ -4532,7 +4533,7 @@
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
@@ -4554,7 +4555,7 @@
       </c>
       <c r="B70" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C70" s="7" t="inlineStr">
@@ -4576,7 +4577,7 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -4598,7 +4599,7 @@
       </c>
       <c r="B72" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C72" s="7" t="inlineStr">
@@ -4620,7 +4621,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
@@ -4642,7 +4643,7 @@
       </c>
       <c r="B74" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C74" s="7" t="inlineStr">
@@ -4664,7 +4665,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -4686,7 +4687,7 @@
       </c>
       <c r="B76" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C76" s="7" t="inlineStr">
@@ -4708,7 +4709,7 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
@@ -4730,7 +4731,7 @@
       </c>
       <c r="B78" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C78" s="7" t="inlineStr">
@@ -4752,7 +4753,7 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
@@ -4774,12 +4775,12 @@
       </c>
       <c r="B80" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C80" s="7" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>reception@fabrikam.example</t>
         </is>
       </c>
       <c r="D80" s="7" t="inlineStr">
@@ -4796,12 +4797,12 @@
       </c>
       <c r="B81" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C81" s="7" t="inlineStr">
         <is>
-          <t>ruby.davies@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D81" s="7" t="inlineStr">
@@ -4818,12 +4819,12 @@
       </c>
       <c r="B82" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C82" s="7" t="inlineStr">
         <is>
-          <t>ruby.wood@fabrikam.example</t>
+          <t>ruby.davies@fabrikam.example</t>
         </is>
       </c>
       <c r="D82" s="7" t="inlineStr">
@@ -4840,12 +4841,12 @@
       </c>
       <c r="B83" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C83" s="7" t="inlineStr">
         <is>
-          <t>thomas.johnson@fabrikam.example</t>
+          <t>ruby.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D83" s="7" t="inlineStr">
@@ -4862,12 +4863,12 @@
       </c>
       <c r="B84" s="7" t="inlineStr">
         <is>
-          <t>27 users without MFA</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C84" s="7" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>thomas.johnson@fabrikam.example</t>
         </is>
       </c>
       <c r="D84" s="7" t="inlineStr">
@@ -4879,22 +4880,22 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Legacy authentication is allowed</t>
+          <t>28 users without MFA</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D85" s="7" t="inlineStr">
         <is>
-          <t>No enabled policy blocks legacy authentication for all users</t>
+          <t>No MFA method registered</t>
         </is>
       </c>
     </row>
@@ -4906,17 +4907,17 @@
       </c>
       <c r="B86" s="7" t="inlineStr">
         <is>
-          <t>1 domain had sign-in settings changed in the last 30 days</t>
+          <t>Legacy authentication is allowed</t>
         </is>
       </c>
       <c r="C86" s="7" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D86" s="7" t="inlineStr">
         <is>
-          <t>Set domain authentication by mallory.quinn@fabrikam.example on 14 Oct 2026</t>
+          <t>No enabled policy blocks legacy authentication for all users</t>
         </is>
       </c>
     </row>
@@ -4928,17 +4929,17 @@
       </c>
       <c r="B87" s="7" t="inlineStr">
         <is>
-          <t>2 sites with no owner, 2 sites with one owner</t>
+          <t>1 domain had sign-in settings changed in the last 30 days</t>
         </is>
       </c>
       <c r="C87" s="7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D87" s="7" t="inlineStr">
         <is>
-          <t>No enabled owner (Microsoft 365 group)</t>
+          <t>Set domain authentication by mallory.quinn@fabrikam.example on 14 Oct 2026</t>
         </is>
       </c>
     </row>
@@ -4955,19 +4956,19 @@
       </c>
       <c r="C88" s="7" t="inlineStr">
         <is>
-          <t>Old Projects</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D88" s="7" t="inlineStr">
         <is>
-          <t>No enabled owner (site administrators and owners group)</t>
+          <t>No enabled owner (Microsoft 365 group)</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -4977,12 +4978,12 @@
       </c>
       <c r="C89" s="7" t="inlineStr">
         <is>
-          <t>Practice Management</t>
+          <t>Old Projects</t>
         </is>
       </c>
       <c r="D89" s="7" t="inlineStr">
         <is>
-          <t>One owner (Microsoft 365 group)</t>
+          <t>No enabled owner (site administrators and owners group)</t>
         </is>
       </c>
     </row>
@@ -4999,34 +5000,34 @@
       </c>
       <c r="C90" s="7" t="inlineStr">
         <is>
-          <t>Staff Intranet</t>
+          <t>Practice Management</t>
         </is>
       </c>
       <c r="D90" s="7" t="inlineStr">
         <is>
-          <t>One owner (site administrators and owners group)</t>
+          <t>One owner (Microsoft 365 group)</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>1 guest with full control of 1 site</t>
+          <t>2 sites with no owner, 2 sites with one owner</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>accounts@hollis-partners.example on Finance</t>
+          <t>Staff Intranet</t>
         </is>
       </c>
       <c r="D91" s="7" t="inlineStr">
         <is>
-          <t>Full Control, given Full Control directly</t>
+          <t>One owner (site administrators and owners group)</t>
         </is>
       </c>
     </row>
@@ -5038,24 +5039,24 @@
       </c>
       <c r="B92" s="7" t="inlineStr">
         <is>
-          <t>2 high or medium severity alerts open in Defender, 1 not picked up</t>
+          <t>1 guest with full control of 1 site</t>
         </is>
       </c>
       <c r="C92" s="7" t="inlineStr">
         <is>
-          <t>Email messages containing malicious URL removed after delivery</t>
+          <t>accounts@hollis-partners.example on Finance</t>
         </is>
       </c>
       <c r="D92" s="7" t="inlineStr">
         <is>
-          <t>Defender for Office 365, nobody has picked it up, since 14 Oct 2026; names anna.kowalski@fabrikam.example</t>
+          <t>Full Control, given Full Control directly</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="B93" s="7" t="inlineStr">
@@ -5065,12 +5066,12 @@
       </c>
       <c r="C93" s="7" t="inlineStr">
         <is>
-          <t>Suspicious PowerShell command line</t>
+          <t>Email messages containing malicious URL removed after delivery</t>
         </is>
       </c>
       <c r="D93" s="7" t="inlineStr">
         <is>
-          <t>Defender for Endpoint, in progress with helpdesk@msp.example, since 12 Oct 2026; names LAPTOP-OKAFOR\bob, LAPTOP-OKAFOR</t>
+          <t>Defender for Office 365, nobody has picked it up, since 15 Oct 2026; names anna.kowalski@fabrikam.example</t>
         </is>
       </c>
     </row>
@@ -5082,17 +5083,17 @@
       </c>
       <c r="B94" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>2 high or medium severity alerts open in Defender, 1 not picked up</t>
         </is>
       </c>
       <c r="C94" s="7" t="inlineStr">
         <is>
-          <t>aaron.smith@fabrikam.example</t>
+          <t>Suspicious PowerShell command line</t>
         </is>
       </c>
       <c r="D94" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 27 Apr 2026</t>
+          <t>Defender for Endpoint, in progress with helpdesk@msp.example, since 13 Oct 2026; names LAPTOP-OKAFOR\bob, LAPTOP-OKAFOR</t>
         </is>
       </c>
     </row>
@@ -5104,17 +5105,17 @@
       </c>
       <c r="B95" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C95" s="7" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>aaron.smith@fabrikam.example</t>
         </is>
       </c>
       <c r="D95" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 11 Mar 2026</t>
+          <t>Licensed member, last signed in 28 Apr 2026</t>
         </is>
       </c>
     </row>
@@ -5126,17 +5127,17 @@
       </c>
       <c r="B96" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C96" s="7" t="inlineStr">
         <is>
-          <t>jack.lee@fabrikam.example</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D96" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 8 Jun 2026</t>
+          <t>Licensed member, last signed in 12 Mar 2026</t>
         </is>
       </c>
     </row>
@@ -5148,17 +5149,17 @@
       </c>
       <c r="B97" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C97" s="7" t="inlineStr">
         <is>
-          <t>noah.wood@fabrikam.example</t>
+          <t>jack.lee@fabrikam.example</t>
         </is>
       </c>
       <c r="D97" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 11 Feb 2026</t>
+          <t>Licensed member, last signed in 9 Jun 2026</t>
         </is>
       </c>
     </row>
@@ -5170,17 +5171,17 @@
       </c>
       <c r="B98" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C98" s="7" t="inlineStr">
         <is>
-          <t>rhys.walker@fabrikam.example</t>
+          <t>noah.wood@fabrikam.example</t>
         </is>
       </c>
       <c r="D98" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 9 Jun 2026</t>
+          <t>Licensed member, last signed in 12 Feb 2026</t>
         </is>
       </c>
     </row>
@@ -5192,83 +5193,83 @@
       </c>
       <c r="B99" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C99" s="7" t="inlineStr">
         <is>
-          <t>zara.edwards@fabrikam.example</t>
+          <t>rhys.walker@fabrikam.example</t>
         </is>
       </c>
       <c r="D99" s="7" t="inlineStr">
         <is>
-          <t>Licensed member, last signed in 13 Jul 2026</t>
+          <t>Licensed member, last signed in 10 Jun 2026</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B100" s="7" t="inlineStr">
         <is>
-          <t>7 accounts inactive for 90+ days or never used</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C100" s="7" t="inlineStr">
         <is>
-          <t>g#EXT#@fabrikam.example</t>
+          <t>zara.edwards@fabrikam.example</t>
         </is>
       </c>
       <c r="D100" s="7" t="inlineStr">
         <is>
-          <t>Guest, never signed in, created ?</t>
+          <t>Licensed member, last signed in 14 Jul 2026</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B101" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C101" s="7" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>reception@fabrikam.example</t>
         </is>
       </c>
       <c r="D101" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with Authenticator app</t>
+          <t>Member, never signed in, created 4 Mar 2024</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B102" s="7" t="inlineStr">
         <is>
-          <t>2 admins without a phishing-resistant method</t>
+          <t>8 accounts inactive for 90+ days or never used</t>
         </is>
       </c>
       <c r="C102" s="7" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>sam.carter_consultants.example#EXT#@fabrikam.onmicrosoft.com</t>
         </is>
       </c>
       <c r="D102" s="7" t="inlineStr">
         <is>
-          <t>Global Administrator; signs in with no MFA method at all</t>
+          <t>Guest, never signed in, created 2 Sep 2025</t>
         </is>
       </c>
     </row>
@@ -5280,17 +5281,17 @@
       </c>
       <c r="B103" s="7" t="inlineStr">
         <is>
-          <t>1 app with privileged roles</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C103" s="7" t="inlineStr">
         <is>
-          <t>Some app</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D103" s="7" t="inlineStr">
         <is>
-          <t>App holding Exchange Administrator</t>
+          <t>Global Administrator; signs in with Authenticator app</t>
         </is>
       </c>
     </row>
@@ -5302,17 +5303,17 @@
       </c>
       <c r="B104" s="7" t="inlineStr">
         <is>
-          <t>Users can consent to any app</t>
+          <t>2 admins without a phishing-resistant method</t>
         </is>
       </c>
       <c r="C104" s="7" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D104" s="7" t="inlineStr">
         <is>
-          <t>Any user can grant any app access to their mail and files</t>
+          <t>Global Administrator; signs in with no MFA method at all</t>
         </is>
       </c>
     </row>
@@ -5324,17 +5325,17 @@
       </c>
       <c r="B105" s="7" t="inlineStr">
         <is>
-          <t>No compliance policy for iOS/iPadOS</t>
+          <t>1 app with privileged roles</t>
         </is>
       </c>
       <c r="C105" s="7" t="inlineStr">
         <is>
-          <t>iOS/iPadOS</t>
+          <t>Backup connector</t>
         </is>
       </c>
       <c r="D105" s="7" t="inlineStr">
         <is>
-          <t>1 enrolled device, no compliance policy assigned</t>
+          <t>App holding Exchange Administrator</t>
         </is>
       </c>
     </row>
@@ -5346,17 +5347,17 @@
       </c>
       <c r="B106" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>Users can consent to any app</t>
         </is>
       </c>
       <c r="C106" s="7" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D106" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>Any user can grant any app access to their mail and files</t>
         </is>
       </c>
     </row>
@@ -5368,17 +5369,17 @@
       </c>
       <c r="B107" s="7" t="inlineStr">
         <is>
-          <t>9 of 55 managed devices not compliant</t>
+          <t>No compliance policy for iOS/iPadOS</t>
         </is>
       </c>
       <c r="C107" s="7" t="inlineStr">
         <is>
-          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
+          <t>iOS/iPadOS</t>
         </is>
       </c>
       <c r="D107" s="7" t="inlineStr">
         <is>
-          <t>Not compliant</t>
+          <t>1 enrolled device, no compliance policy assigned</t>
         </is>
       </c>
     </row>
@@ -5395,17 +5396,12 @@
       </c>
       <c r="C108" s="7" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D108" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
-        </is>
-      </c>
-      <c r="E108" t="inlineStr">
-        <is>
-          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5422,7 +5418,7 @@
       </c>
       <c r="C109" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-MOORE18 (ava.moore@fabrikam.example)</t>
         </is>
       </c>
       <c r="D109" s="7" t="inlineStr">
@@ -5444,12 +5440,17 @@
       </c>
       <c r="C110" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D110" s="7" t="inlineStr">
         <is>
           <t>Not compliant</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -5466,7 +5467,7 @@
       </c>
       <c r="C111" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D111" s="7" t="inlineStr">
@@ -5488,7 +5489,7 @@
       </c>
       <c r="C112" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D112" s="7" t="inlineStr">
@@ -5510,7 +5511,7 @@
       </c>
       <c r="C113" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D113" s="7" t="inlineStr">
@@ -5532,7 +5533,7 @@
       </c>
       <c r="C114" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
+          <t>LAPTOP-ROBINSON07 (thomas.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D114" s="7" t="inlineStr">
@@ -5549,17 +5550,17 @@
       </c>
       <c r="B115" s="7" t="inlineStr">
         <is>
-          <t>7 of 55 joined Windows computers without a saved recovery key</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C115" s="7" t="inlineStr">
         <is>
-          <t>DESK-SMITH03</t>
+          <t>LAPTOP-WARD29 (jack.ward@fabrikam.example)</t>
         </is>
       </c>
       <c r="D115" s="7" t="inlineStr">
         <is>
-          <t>Encrypted, but no recovery key saved in Entra ID</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -5571,17 +5572,17 @@
       </c>
       <c r="B116" s="7" t="inlineStr">
         <is>
-          <t>7 of 55 joined Windows computers without a saved recovery key</t>
+          <t>9 of 55 managed devices not compliant</t>
         </is>
       </c>
       <c r="C116" s="7" t="inlineStr">
         <is>
-          <t>DESK-WHITE42</t>
+          <t>LAPTOP-WATSON40 (lily.watson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D116" s="7" t="inlineStr">
         <is>
-          <t>Encrypted, but no recovery key saved in Entra ID</t>
+          <t>Not compliant</t>
         </is>
       </c>
     </row>
@@ -5598,7 +5599,7 @@
       </c>
       <c r="C117" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-EVANS26</t>
+          <t>DESK-SMITH03</t>
         </is>
       </c>
       <c r="D117" s="7" t="inlineStr">
@@ -5620,7 +5621,7 @@
       </c>
       <c r="C118" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-HUGHES11</t>
+          <t>DESK-WHITE42</t>
         </is>
       </c>
       <c r="D118" s="7" t="inlineStr">
@@ -5642,7 +5643,7 @@
       </c>
       <c r="C119" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-JACKSON49</t>
+          <t>LAPTOP-EVANS26</t>
         </is>
       </c>
       <c r="D119" s="7" t="inlineStr">
@@ -5664,7 +5665,7 @@
       </c>
       <c r="C120" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-JONES34</t>
+          <t>LAPTOP-HUGHES11</t>
         </is>
       </c>
       <c r="D120" s="7" t="inlineStr">
@@ -5686,7 +5687,7 @@
       </c>
       <c r="C121" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-SCOTT19</t>
+          <t>LAPTOP-JACKSON49</t>
         </is>
       </c>
       <c r="D121" s="7" t="inlineStr">
@@ -5703,17 +5704,17 @@
       </c>
       <c r="B122" s="7" t="inlineStr">
         <is>
-          <t>1 mail domain without DKIM</t>
+          <t>7 of 55 joined Windows computers without a saved recovery key</t>
         </is>
       </c>
       <c r="C122" s="7" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-JONES34</t>
         </is>
       </c>
       <c r="D122" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
+          <t>Encrypted, but no recovery key saved in Entra ID</t>
         </is>
       </c>
     </row>
@@ -5725,39 +5726,39 @@
       </c>
       <c r="B123" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>7 of 55 joined Windows computers without a saved recovery key</t>
         </is>
       </c>
       <c r="C123" s="7" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-SCOTT19</t>
         </is>
       </c>
       <c r="D123" s="7" t="inlineStr">
         <is>
-          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
+          <t>Encrypted, but no recovery key saved in Entra ID</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B124" s="7" t="inlineStr">
         <is>
-          <t>2 domains without DMARC enforcement</t>
+          <t>1 mail domain without DKIM</t>
         </is>
       </c>
       <c r="C124" s="7" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D124" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no DMARC p=reject record</t>
+          <t>Microsoft 365 DKIM isn't set up (selector2 CNAME missing)</t>
         </is>
       </c>
     </row>
@@ -5769,39 +5770,39 @@
       </c>
       <c r="B125" s="7" t="inlineStr">
         <is>
-          <t>1 anti-malware policy lets risky attachment types through</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C125" s="7" t="inlineStr">
         <is>
-          <t>Default</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D125" s="7" t="inlineStr">
         <is>
-          <t>The common attachments filter is off</t>
+          <t>DMARC is monitor-only (p=none); spoofed mail is still delivered</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B126" s="7" t="inlineStr">
         <is>
-          <t>1 anti-phishing policy weakens spoof protection</t>
+          <t>2 domains without DMARC enforcement</t>
         </is>
       </c>
       <c r="C126" s="7" t="inlineStr">
         <is>
-          <t>Office365 AntiPhish Default</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D126" s="7" t="inlineStr">
         <is>
-          <t>Ignores what senders' DMARC policies ask for</t>
+          <t>Needs a DMARC p=reject record, or spoofed mail from it is still delivered</t>
         </is>
       </c>
     </row>
@@ -5813,68 +5814,68 @@
       </c>
       <c r="B127" s="7" t="inlineStr">
         <is>
-          <t>4 teams and groups without an owner</t>
+          <t>1 anti-malware policy lets risky attachment types through</t>
         </is>
       </c>
       <c r="C127" s="7" t="inlineStr">
         <is>
-          <t>Project Phoenix</t>
+          <t>Default</t>
         </is>
       </c>
       <c r="D127" s="7" t="inlineStr">
         <is>
-          <t>Team, only owner is disabled (Ben Okafor)</t>
+          <t>The common attachments filter is off</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B128" s="7" t="inlineStr">
         <is>
-          <t>4 teams and groups without an owner</t>
+          <t>1 of 3 shared mailboxes allows sign-in</t>
         </is>
       </c>
       <c r="C128" s="7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>reception@fabrikam.example</t>
         </is>
       </c>
       <c r="D128" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, only owner is disabled (Ben Okafor)</t>
+          <t>Shared mailbox account allows sign-in</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B129" s="7" t="inlineStr">
         <is>
-          <t>4 teams and groups without an owner</t>
+          <t>1 anti-phishing policy weakens spoof protection</t>
         </is>
       </c>
       <c r="C129" s="7" t="inlineStr">
         <is>
-          <t>Marketing</t>
+          <t>Office365 AntiPhish Default</t>
         </is>
       </c>
       <c r="D129" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, no owner</t>
+          <t>Ignores what senders' DMARC policies ask for</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B130" s="7" t="inlineStr">
@@ -5884,78 +5885,78 @@
       </c>
       <c r="C130" s="7" t="inlineStr">
         <is>
-          <t>Provisioned</t>
+          <t>Project Phoenix</t>
         </is>
       </c>
       <c r="D130" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
+          <t>Team, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B131" s="7" t="inlineStr">
         <is>
-          <t>Enforced by CA002 — All users: Require MFA, with 1 exclusion to review</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C131" s="7" t="inlineStr">
         <is>
-          <t>breakglass@fabrikam.example</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D131" s="7" t="inlineStr">
         <is>
-          <t>Excluded from "CA002 — All users: Require MFA"</t>
+          <t>Microsoft 365 group, only owner is disabled (Ben Okafor)</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B132" s="7" t="inlineStr">
         <is>
-          <t>1 disabled account still licensed</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C132" s="7" t="inlineStr">
         <is>
-          <t>ben.okafor@fabrikam.example</t>
+          <t>Marketing</t>
         </is>
       </c>
       <c r="D132" s="7" t="inlineStr">
         <is>
-          <t>Disabled, holding 1 licence</t>
+          <t>Microsoft 365 group, no owner</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="B133" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including anonymous links</t>
+          <t>4 teams and groups without an owner</t>
         </is>
       </c>
       <c r="C133" s="7" t="inlineStr">
         <is>
-          <t>SharePoint and OneDrive</t>
+          <t>Provisioned</t>
         </is>
       </c>
       <c r="D133" s="7" t="inlineStr">
         <is>
-          <t>Anyone links are allowed</t>
+          <t>Microsoft 365 group, owned only by an app (Provisioning app)</t>
         </is>
       </c>
     </row>
@@ -5967,17 +5968,17 @@
       </c>
       <c r="B134" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>Enforced by CA002 — All users: Require MFA, with 1 exclusion to review</t>
         </is>
       </c>
       <c r="C134" s="7" t="inlineStr">
         <is>
-          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
+          <t>breakglass@fabrikam.example</t>
         </is>
       </c>
       <c r="D134" s="7" t="inlineStr">
         <is>
-          <t>Anyone can view</t>
+          <t>Excluded from "CA002 — All users: Require MFA"</t>
         </is>
       </c>
     </row>
@@ -5989,17 +5990,17 @@
       </c>
       <c r="B135" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders shared with anyone</t>
+          <t>1 disabled account still licensed (not counting 1 shared mailbox that needs one)</t>
         </is>
       </c>
       <c r="C135" s="7" t="inlineStr">
         <is>
-          <t>Open day flyer.pdf (Marketing / Documents)</t>
+          <t>ben.okafor@fabrikam.example</t>
         </is>
       </c>
       <c r="D135" s="7" t="inlineStr">
         <is>
-          <t>Anyone can view, link never expires</t>
+          <t>Disabled, holding 1 licence</t>
         </is>
       </c>
     </row>
@@ -6011,22 +6012,17 @@
       </c>
       <c r="B136" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders outside people can edit</t>
+          <t>Anyone, including anonymous links</t>
         </is>
       </c>
       <c r="C136" s="7" t="inlineStr">
         <is>
-          <t>Budget.xlsx (Finance / Documents)</t>
+          <t>SharePoint and OneDrive</t>
         </is>
       </c>
       <c r="D136" s="7" t="inlineStr">
         <is>
-          <t>Can be edited by accountant@hargreaves-partners.example</t>
-        </is>
-      </c>
-      <c r="E136" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Anyone links are allowed</t>
         </is>
       </c>
     </row>
@@ -6038,17 +6034,17 @@
       </c>
       <c r="B137" s="7" t="inlineStr">
         <is>
-          <t>2 files and folders outside people can edit</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C137" s="7" t="inlineStr">
         <is>
-          <t>Lab dockets (Patient Records / Documents)</t>
+          <t>holiday.jpg (OneDrive of anna.kowalski@fabrikam.example)</t>
         </is>
       </c>
       <c r="D137" s="7" t="inlineStr">
         <is>
-          <t>Can be edited by orders@dentallab.example</t>
+          <t>Anyone can view</t>
         </is>
       </c>
     </row>
@@ -6060,17 +6056,17 @@
       </c>
       <c r="B138" s="7" t="inlineStr">
         <is>
-          <t>3 mailboxes at or over 90% of quota</t>
+          <t>2 files and folders shared with anyone</t>
         </is>
       </c>
       <c r="C138" s="7" t="inlineStr">
         <is>
-          <t>accounts@fabrikam.example</t>
+          <t>Open day flyer.pdf (Marketing / Documents)</t>
         </is>
       </c>
       <c r="D138" s="7" t="inlineStr">
         <is>
-          <t>44.8 GB of 49.5 GB (91%), no archive</t>
+          <t>Anyone can view, link never expires</t>
         </is>
       </c>
     </row>
@@ -6082,17 +6078,17 @@
       </c>
       <c r="B139" s="7" t="inlineStr">
         <is>
-          <t>3 mailboxes at or over 90% of quota</t>
+          <t>2 files and folders outside people can edit</t>
         </is>
       </c>
       <c r="C139" s="7" t="inlineStr">
         <is>
-          <t>aisha.brown@fabrikam.example</t>
+          <t>Budget.xlsx (Finance / Documents)</t>
         </is>
       </c>
       <c r="D139" s="7" t="inlineStr">
         <is>
-          <t>47.2 GB of 49.5 GB (95%), no archive</t>
+          <t>Can be edited by accountant@hargreaves-partners.example</t>
         </is>
       </c>
       <c r="E139" t="inlineStr">
@@ -6109,22 +6105,17 @@
       </c>
       <c r="B140" s="7" t="inlineStr">
         <is>
-          <t>3 mailboxes at or over 90% of quota</t>
+          <t>2 files and folders outside people can edit</t>
         </is>
       </c>
       <c r="C140" s="7" t="inlineStr">
         <is>
-          <t>thomas.robinson@fabrikam.example</t>
+          <t>Lab dockets (Patient Records / Documents)</t>
         </is>
       </c>
       <c r="D140" s="7" t="inlineStr">
         <is>
-          <t>45.6 GB of 49.5 GB (92%), no archive</t>
-        </is>
-      </c>
-      <c r="E140" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Can be edited by orders@dentallab.example</t>
         </is>
       </c>
     </row>
@@ -6136,44 +6127,39 @@
       </c>
       <c r="B141" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C141" s="7" t="inlineStr">
         <is>
-          <t>Tenant SharePoint storage</t>
+          <t>accounts@fabrikam.example</t>
         </is>
       </c>
       <c r="D141" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
-        </is>
-      </c>
-      <c r="E141" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>44.8 GB of 49.5 GB (91%), no archive</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B142" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C142" s="7" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/finance</t>
+          <t>aisha.brown@fabrikam.example</t>
         </is>
       </c>
       <c r="D142" s="7" t="inlineStr">
         <is>
-          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
+          <t>47.2 GB of 49.5 GB (95%), no archive</t>
         </is>
       </c>
       <c r="E142" t="inlineStr">
@@ -6185,22 +6171,22 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B143" s="7" t="inlineStr">
         <is>
-          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
+          <t>3 mailboxes at or over 90% of quota</t>
         </is>
       </c>
       <c r="C143" s="7" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
+          <t>thomas.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D143" s="7" t="inlineStr">
         <is>
-          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
+          <t>45.6 GB of 49.5 GB (92%), no archive</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
@@ -6212,7 +6198,7 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="B144" s="7" t="inlineStr">
@@ -6222,12 +6208,12 @@
       </c>
       <c r="C144" s="7" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
+          <t>Tenant SharePoint storage</t>
         </is>
       </c>
       <c r="D144" s="7" t="inlineStr">
         <is>
-          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="E144" t="inlineStr">
@@ -6249,12 +6235,12 @@
       </c>
       <c r="C145" s="7" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
+          <t>https://fabrikam.sharepoint.com/sites/finance</t>
         </is>
       </c>
       <c r="D145" s="7" t="inlineStr">
         <is>
-          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
+          <t>117.5 GB, of which 3.0 GB in the recycle bin and 7.6 GB older versions</t>
         </is>
       </c>
       <c r="E145" t="inlineStr">
@@ -6276,12 +6262,12 @@
       </c>
       <c r="C146" s="7" t="inlineStr">
         <is>
-          <t>https://fabrikam.sharepoint.com/sites/practice</t>
+          <t>https://fabrikam.sharepoint.com/sites/imaging</t>
         </is>
       </c>
       <c r="D146" s="7" t="inlineStr">
         <is>
-          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+          <t>483.2 GB, of which 46.0 GB in the recycle bin and 33.3 GB older versions</t>
         </is>
       </c>
       <c r="E146" t="inlineStr">
@@ -6298,17 +6284,22 @@
       </c>
       <c r="B147" s="7" t="inlineStr">
         <is>
-          <t>1 account reports to a blocked manager</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C147" s="7" t="inlineStr">
         <is>
-          <t>anna.kowalski@fabrikam.example</t>
+          <t>https://fabrikam.sharepoint.com/sites/marketing</t>
         </is>
       </c>
       <c r="D147" s="7" t="inlineStr">
         <is>
-          <t>Reports to Ben Okafor, whose sign-in is blocked</t>
+          <t>65.3 GB, of which 1.0 GB in the recycle bin and 4.9 GB older versions</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6320,17 +6311,22 @@
       </c>
       <c r="B148" s="7" t="inlineStr">
         <is>
-          <t>1 app registration with expiring or expired credentials</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C148" s="7" t="inlineStr">
         <is>
-          <t>Old connector</t>
+          <t>https://fabrikam.sharepoint.com/sites/patient-records</t>
         </is>
       </c>
       <c r="D148" s="7" t="inlineStr">
         <is>
-          <t>The 1 credential expired, last on 1 Jan 2025</t>
+          <t>352.6 GB, of which 12.0 GB in the recycle bin and 25.2 GB older versions</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6342,17 +6338,22 @@
       </c>
       <c r="B149" s="7" t="inlineStr">
         <is>
-          <t>1 of 55 joined computers not in Intune</t>
+          <t>88% of about 1.45 TB used (1 TB + 10 GB × 46 licences)</t>
         </is>
       </c>
       <c r="C149" s="7" t="inlineStr">
         <is>
-          <t>DESK-RECEPTION</t>
+          <t>https://fabrikam.sharepoint.com/sites/practice</t>
         </is>
       </c>
       <c r="D149" s="7" t="inlineStr">
         <is>
-          <t>Hybrid joined, not managed by Intune</t>
+          <t>182.8 GB, of which 6.0 GB in the recycle bin and 21.1 GB older versions</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6364,17 +6365,17 @@
       </c>
       <c r="B150" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 account reports to a blocked manager</t>
         </is>
       </c>
       <c r="C150" s="7" t="inlineStr">
         <is>
-          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
+          <t>anna.kowalski@fabrikam.example</t>
         </is>
       </c>
       <c r="D150" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>Reports to Ben Okafor, whose sign-in is blocked</t>
         </is>
       </c>
     </row>
@@ -6386,22 +6387,17 @@
       </c>
       <c r="B151" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 app registration with expiring or expired credentials</t>
         </is>
       </c>
       <c r="C151" s="7" t="inlineStr">
         <is>
-          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
+          <t>Old connector</t>
         </is>
       </c>
       <c r="D151" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
-        </is>
-      </c>
-      <c r="E151" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>The 1 credential expired, last on 1 Jan 2025</t>
         </is>
       </c>
     </row>
@@ -6413,17 +6409,17 @@
       </c>
       <c r="B152" s="7" t="inlineStr">
         <is>
-          <t>5 devices haven't checked in for 30+ days</t>
+          <t>1 of 55 joined computers not in Intune</t>
         </is>
       </c>
       <c r="C152" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
+          <t>DESK-RECEPTION</t>
         </is>
       </c>
       <c r="D152" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 38 days ago</t>
+          <t>Hybrid joined, not managed by Intune</t>
         </is>
       </c>
     </row>
@@ -6440,7 +6436,7 @@
       </c>
       <c r="C153" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
+          <t>DESK-LEWIS12 (william.lewis@fabrikam.example)</t>
         </is>
       </c>
       <c r="D153" s="7" t="inlineStr">
@@ -6462,12 +6458,17 @@
       </c>
       <c r="C154" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
+          <t>DESK-ROBINSON51 (owen.robinson@fabrikam.example)</t>
         </is>
       </c>
       <c r="D154" s="7" t="inlineStr">
         <is>
-          <t>Last check-in 45 days ago</t>
+          <t>Last check-in 38 days ago</t>
+        </is>
+      </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6479,17 +6480,17 @@
       </c>
       <c r="B155" s="7" t="inlineStr">
         <is>
-          <t>1 of 57 device records unused for 90+ days</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C155" s="7" t="inlineStr">
         <is>
-          <t>OLD-PC</t>
+          <t>LAPTOP-DAVIES38 (ruby.davies@fabrikam.example)</t>
         </is>
       </c>
       <c r="D155" s="7" t="inlineStr">
         <is>
-          <t>Windows, last seen 200 days ago</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -6501,17 +6502,17 @@
       </c>
       <c r="B156" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C156" s="7" t="inlineStr">
         <is>
-          <t>DESK-HARRISON21</t>
+          <t>LAPTOP-LEE25 (arthur.lee@fabrikam.example)</t>
         </is>
       </c>
       <c r="D156" s="7" t="inlineStr">
         <is>
-          <t>No local admin password backed up in Entra ID</t>
+          <t>Last check-in 38 days ago</t>
         </is>
       </c>
     </row>
@@ -6523,17 +6524,17 @@
       </c>
       <c r="B157" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
+          <t>5 devices haven't checked in for 30+ days</t>
         </is>
       </c>
       <c r="C157" s="7" t="inlineStr">
         <is>
-          <t>DESK-ROBERTS45</t>
+          <t>LAPTOP-OKAFOR (ben.okafor@fabrikam.example)</t>
         </is>
       </c>
       <c r="D157" s="7" t="inlineStr">
         <is>
-          <t>No local admin password backed up in Entra ID</t>
+          <t>Last check-in 45 days ago</t>
         </is>
       </c>
     </row>
@@ -6545,17 +6546,17 @@
       </c>
       <c r="B158" s="7" t="inlineStr">
         <is>
-          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
+          <t>1 of 57 device records unused for 90+ days</t>
         </is>
       </c>
       <c r="C158" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-SMITH13</t>
+          <t>OLD-PC</t>
         </is>
       </c>
       <c r="D158" s="7" t="inlineStr">
         <is>
-          <t>No local admin password backed up in Entra ID</t>
+          <t>Windows, last seen 200 days ago</t>
         </is>
       </c>
     </row>
@@ -6572,7 +6573,7 @@
       </c>
       <c r="C159" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-TURNER37</t>
+          <t>DESK-HARRISON21</t>
         </is>
       </c>
       <c r="D159" s="7" t="inlineStr">
@@ -6594,7 +6595,7 @@
       </c>
       <c r="C160" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-WARD29</t>
+          <t>DESK-ROBERTS45</t>
         </is>
       </c>
       <c r="D160" s="7" t="inlineStr">
@@ -6616,7 +6617,7 @@
       </c>
       <c r="C161" s="7" t="inlineStr">
         <is>
-          <t>LAPTOP-WOOD05</t>
+          <t>LAPTOP-SMITH13</t>
         </is>
       </c>
       <c r="D161" s="7" t="inlineStr">
@@ -6633,17 +6634,17 @@
       </c>
       <c r="B162" s="7" t="inlineStr">
         <is>
-          <t>1 domain with SPF problems</t>
+          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
         </is>
       </c>
       <c r="C162" s="7" t="inlineStr">
         <is>
-          <t>parked.example</t>
+          <t>LAPTOP-TURNER37</t>
         </is>
       </c>
       <c r="D162" s="7" t="inlineStr">
         <is>
-          <t>Doesn't receive mail but has no "v=spf1 -all" record to stop spoofing</t>
+          <t>No local admin password backed up in Entra ID</t>
         </is>
       </c>
     </row>
@@ -6655,17 +6656,17 @@
       </c>
       <c r="B163" s="7" t="inlineStr">
         <is>
-          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
+          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
         </is>
       </c>
       <c r="C163" s="7" t="inlineStr">
         <is>
-          <t>fabrikam.example</t>
+          <t>LAPTOP-WARD29</t>
         </is>
       </c>
       <c r="D163" s="7" t="inlineStr">
         <is>
-          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
+          <t>No local admin password backed up in Entra ID</t>
         </is>
       </c>
     </row>
@@ -6677,17 +6678,17 @@
       </c>
       <c r="B164" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is on for the organisation</t>
+          <t>6 of 54 Entra joined Windows computers without a LAPS backup</t>
         </is>
       </c>
       <c r="C164" s="7" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>LAPTOP-WOOD05</t>
         </is>
       </c>
       <c r="D164" s="7" t="inlineStr">
         <is>
-          <t>SMTP AUTH is allowed</t>
+          <t>No local admin password backed up in Entra ID</t>
         </is>
       </c>
     </row>
@@ -6699,17 +6700,17 @@
       </c>
       <c r="B165" s="7" t="inlineStr">
         <is>
-          <t>Anyone, including guests, can invite guests</t>
+          <t>1 domain with SPF problems</t>
         </is>
       </c>
       <c r="C165" s="7" t="inlineStr">
         <is>
-          <t>Whole organisation</t>
+          <t>parked.example</t>
         </is>
       </c>
       <c r="D165" s="7" t="inlineStr">
         <is>
-          <t>Guests can invite other guests</t>
+          <t>Needs a "v=spf1 -all" record saying it sends no mail, or anyone can send as it</t>
         </is>
       </c>
     </row>
@@ -6721,17 +6722,17 @@
       </c>
       <c r="B166" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>1 of 1 mail domain doesn't fully enforce MTA-STS</t>
         </is>
       </c>
       <c r="C166" s="7" t="inlineStr">
         <is>
-          <t>george.baker@fabrikam.example</t>
+          <t>fabrikam.example</t>
         </is>
       </c>
       <c r="D166" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>No MTA-STS policy, so mail sent to this domain can be forced onto an unencrypted connection</t>
         </is>
       </c>
     </row>
@@ -6743,22 +6744,17 @@
       </c>
       <c r="B167" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>SMTP AUTH is on for the organisation</t>
         </is>
       </c>
       <c r="C167" s="7" t="inlineStr">
         <is>
-          <t>owen.robinson@fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D167" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
-        </is>
-      </c>
-      <c r="E167" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>SMTP AUTH is allowed</t>
         </is>
       </c>
     </row>
@@ -6770,17 +6766,17 @@
       </c>
       <c r="B168" s="7" t="inlineStr">
         <is>
-          <t>4 people can only use a text or call as a second factor</t>
+          <t>Anyone, including guests, can invite guests</t>
         </is>
       </c>
       <c r="C168" s="7" t="inlineStr">
         <is>
-          <t>owen.turner@fabrikam.example</t>
+          <t>Whole organisation</t>
         </is>
       </c>
       <c r="D168" s="7" t="inlineStr">
         <is>
-          <t>Second factor is only Mobile phone (SMS or call)</t>
+          <t>Guests can invite other guests</t>
         </is>
       </c>
     </row>
@@ -6797,7 +6793,7 @@
       </c>
       <c r="C169" s="7" t="inlineStr">
         <is>
-          <t>thomas.allen@fabrikam.example</t>
+          <t>george.baker@fabrikam.example</t>
         </is>
       </c>
       <c r="D169" s="7" t="inlineStr">
@@ -6814,17 +6810,22 @@
       </c>
       <c r="B170" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>4 people can only use a text or call as a second factor</t>
         </is>
       </c>
       <c r="C170" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Basic</t>
+          <t>owen.robinson@fabrikam.example</t>
         </is>
       </c>
       <c r="D170" s="7" t="inlineStr">
         <is>
-          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
     </row>
@@ -6836,17 +6837,17 @@
       </c>
       <c r="B171" s="7" t="inlineStr">
         <is>
-          <t>2 subscriptions with spare licences</t>
+          <t>4 people can only use a text or call as a second factor</t>
         </is>
       </c>
       <c r="C171" s="7" t="inlineStr">
         <is>
-          <t>Microsoft 365 Business Premium</t>
+          <t>owen.turner@fabrikam.example</t>
         </is>
       </c>
       <c r="D171" s="7" t="inlineStr">
         <is>
-          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
         </is>
       </c>
     </row>
@@ -6858,22 +6859,88 @@
       </c>
       <c r="B172" s="7" t="inlineStr">
         <is>
+          <t>4 people can only use a text or call as a second factor</t>
+        </is>
+      </c>
+      <c r="C172" s="7" t="inlineStr">
+        <is>
+          <t>thomas.allen@fabrikam.example</t>
+        </is>
+      </c>
+      <c r="D172" s="7" t="inlineStr">
+        <is>
+          <t>Second factor is only Mobile phone (SMS or call)</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B173" s="7" t="inlineStr">
+        <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C173" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Basic</t>
+        </is>
+      </c>
+      <c r="D173" s="7" t="inlineStr">
+        <is>
+          <t>2 of 13 unassigned, 9.80 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B174" s="7" t="inlineStr">
+        <is>
+          <t>2 subscriptions with spare licences</t>
+        </is>
+      </c>
+      <c r="C174" s="7" t="inlineStr">
+        <is>
+          <t>Microsoft 365 Business Premium</t>
+        </is>
+      </c>
+      <c r="D174" s="7" t="inlineStr">
+        <is>
+          <t>3 of 46 unassigned, 54.30 GBP/month</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B175" s="7" t="inlineStr">
+        <is>
           <t>Any user can register an app</t>
         </is>
       </c>
-      <c r="C172" s="7" t="inlineStr">
+      <c r="C175" s="7" t="inlineStr">
         <is>
           <t>Whole organisation</t>
         </is>
       </c>
-      <c r="D172" s="7" t="inlineStr">
+      <c r="D175" s="7" t="inlineStr">
         <is>
           <t>Users can register apps that nobody reviews</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E172"/>
+  <autoFilter ref="A1:E175"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
@@ -6986,10 +7053,10 @@
       <c r="G2" t="n">
         <v>4</v>
       </c>
-      <c r="H2" s="12" t="n">
+      <c r="H2" s="11" t="n">
         <v>18.1</v>
       </c>
-      <c r="I2" s="12" t="n">
+      <c r="I2" s="11" t="n">
         <v>144.8</v>
       </c>
     </row>
@@ -7019,10 +7086,10 @@
       <c r="G3" t="n">
         <v>2</v>
       </c>
-      <c r="H3" s="12" t="n">
+      <c r="H3" s="11" t="n">
         <v>4.9</v>
       </c>
-      <c r="I3" s="12" t="n">
+      <c r="I3" s="11" t="n">
         <v>19.6</v>
       </c>
     </row>
@@ -7078,8 +7145,8 @@
           <t>Tenant profile and licences</t>
         </is>
       </c>
-      <c r="B2" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B2" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -7093,8 +7160,8 @@
           <t>Connection and permissions</t>
         </is>
       </c>
-      <c r="B3" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B3" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -7108,8 +7175,8 @@
           <t>Users</t>
         </is>
       </c>
-      <c r="B4" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B4" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -7123,8 +7190,8 @@
           <t>Admin roles</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B5" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -7138,8 +7205,8 @@
           <t>Conditional Access</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B6" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -7153,8 +7220,8 @@
           <t>MFA registration</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B7" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -7168,8 +7235,8 @@
           <t>Per-user MFA</t>
         </is>
       </c>
-      <c r="B8" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B8" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -7183,8 +7250,8 @@
           <t>Secure Score</t>
         </is>
       </c>
-      <c r="B9" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B9" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -7198,8 +7265,8 @@
           <t>Sign-in methods policy</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B10" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -7213,8 +7280,8 @@
           <t>Admin activity</t>
         </is>
       </c>
-      <c r="B11" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B11" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
@@ -7228,8 +7295,8 @@
           <t>Apps and consents</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B12" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -7243,8 +7310,8 @@
           <t>Sharing and consent settings</t>
         </is>
       </c>
-      <c r="B13" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B13" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -7258,8 +7325,8 @@
           <t>Groups and Teams</t>
         </is>
       </c>
-      <c r="B14" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B14" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -7273,8 +7340,8 @@
           <t>Deleted users and groups</t>
         </is>
       </c>
-      <c r="B15" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B15" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -7288,8 +7355,8 @@
           <t>Mailboxes</t>
         </is>
       </c>
-      <c r="B16" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B16" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -7303,8 +7370,8 @@
           <t>Inbox rules</t>
         </is>
       </c>
-      <c r="B17" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B17" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -7318,8 +7385,8 @@
           <t>Sign-in activity</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B18" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -7333,8 +7400,8 @@
           <t>Mailbox size</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B19" s="12" t="n">
+        <v>46312.42236111111</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -7348,8 +7415,8 @@
           <t>Legacy sign-ins</t>
         </is>
       </c>
-      <c r="B20" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B20" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -7363,8 +7430,8 @@
           <t>Mobile devices</t>
         </is>
       </c>
-      <c r="B21" s="13" t="n">
-        <v>46311.5654050926</v>
+      <c r="B21" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -7378,8 +7445,8 @@
           <t>Automatic replies</t>
         </is>
       </c>
-      <c r="B22" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B22" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -7393,8 +7460,8 @@
           <t>Distribution lists</t>
         </is>
       </c>
-      <c r="B23" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B23" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -7408,8 +7475,8 @@
           <t>Risky users</t>
         </is>
       </c>
-      <c r="B24" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B24" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -7423,8 +7490,8 @@
           <t>Security alerts</t>
         </is>
       </c>
-      <c r="B25" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B25" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -7438,8 +7505,8 @@
           <t>Email domains</t>
         </is>
       </c>
-      <c r="B26" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B26" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -7453,8 +7520,8 @@
           <t>Devices</t>
         </is>
       </c>
-      <c r="B27" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B27" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -7468,8 +7535,8 @@
           <t>Intune policies</t>
         </is>
       </c>
-      <c r="B28" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B28" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -7483,8 +7550,8 @@
           <t>Installed apps</t>
         </is>
       </c>
-      <c r="B29" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B29" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -7498,8 +7565,8 @@
           <t>Directory sync</t>
         </is>
       </c>
-      <c r="B30" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B30" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -7513,8 +7580,8 @@
           <t>SharePoint and OneDrive usage</t>
         </is>
       </c>
-      <c r="B31" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B31" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -7528,8 +7595,8 @@
           <t>Shared files</t>
         </is>
       </c>
-      <c r="B32" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B32" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
@@ -7543,8 +7610,8 @@
           <t>SharePoint storage</t>
         </is>
       </c>
-      <c r="B33" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B33" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
@@ -7558,8 +7625,8 @@
           <t>Site permissions</t>
         </is>
       </c>
-      <c r="B34" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B34" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
@@ -7573,8 +7640,8 @@
           <t>Site access</t>
         </is>
       </c>
-      <c r="B35" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B35" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
@@ -7588,8 +7655,8 @@
           <t>Microsoft 365 usage</t>
         </is>
       </c>
-      <c r="B36" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B36" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -7603,8 +7670,8 @@
           <t>Teams</t>
         </is>
       </c>
-      <c r="B37" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B37" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -7618,8 +7685,8 @@
           <t>Mail flow</t>
         </is>
       </c>
-      <c r="B38" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B38" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -7633,8 +7700,8 @@
           <t>Mail rules and protection</t>
         </is>
       </c>
-      <c r="B39" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B39" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
@@ -7648,8 +7715,8 @@
           <t>App sign-ins</t>
         </is>
       </c>
-      <c r="B40" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B40" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -7663,8 +7730,8 @@
           <t>Group nesting</t>
         </is>
       </c>
-      <c r="B41" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B41" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -7678,8 +7745,8 @@
           <t>Departments and managers</t>
         </is>
       </c>
-      <c r="B42" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B42" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -7693,8 +7760,8 @@
           <t>Administrative units</t>
         </is>
       </c>
-      <c r="B43" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B43" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -7708,8 +7775,8 @@
           <t>Service health</t>
         </is>
       </c>
-      <c r="B44" s="13" t="n">
-        <v>46311.56541666666</v>
+      <c r="B44" s="12" t="n">
+        <v>46312.42237268519</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>

</xml_diff>